<commit_message>
Add 03 Oct 2026 ship movement data, Excel summary and history continuity
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01-10-2026/PAT_Berth_Window.xlsx
+++ b/01-10-2026/PAT_Berth_Window.xlsx
@@ -14,6 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="30 Sep 2026" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 Oct 2026" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 Oct 2026" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 Oct 2026" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -506,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -515,6 +516,7 @@
     <col width="32" customWidth="1" min="4" max="4"/>
     <col width="36" customWidth="1" min="5" max="5"/>
     <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -562,6 +564,11 @@
           <t>02 Oct 2026</t>
         </is>
       </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>03 Oct 2026</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -586,6 +593,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr"/>
       <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -614,6 +622,7 @@
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -634,6 +643,7 @@
       <c r="D7" s="5" t="inlineStr"/>
       <c r="E7" s="5" t="inlineStr"/>
       <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -658,6 +668,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr"/>
       <c r="F8" s="5" t="inlineStr"/>
+      <c r="G8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -682,6 +693,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr"/>
       <c r="F9" s="5" t="inlineStr"/>
+      <c r="G9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -702,6 +714,7 @@
       <c r="D10" s="5" t="inlineStr"/>
       <c r="E10" s="5" t="inlineStr"/>
       <c r="F10" s="5" t="inlineStr"/>
+      <c r="G10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -730,6 +743,7 @@
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr"/>
+      <c r="G11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -750,6 +764,7 @@
       <c r="D12" s="5" t="inlineStr"/>
       <c r="E12" s="5" t="inlineStr"/>
       <c r="F12" s="5" t="inlineStr"/>
+      <c r="G12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -778,6 +793,7 @@
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr"/>
+      <c r="G13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -810,6 +826,11 @@
           <t>alongside · 20AB (ETD now 02/15)</t>
         </is>
       </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>sailed (02/15)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -838,6 +859,7 @@
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr"/>
+      <c r="G15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -866,6 +888,11 @@
           <t>alongside · 20B (marked)</t>
         </is>
       </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>sailed (02/17)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -892,6 +919,11 @@
       <c r="F17" s="6" t="inlineStr">
         <is>
           <t>alongside · 20D (marked, 1C)</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>sailed (02/17)</t>
         </is>
       </c>
     </row>
@@ -918,6 +950,11 @@
           <t>alongside → 20F</t>
         </is>
       </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>alongside · 20F</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -940,6 +977,11 @@
       <c r="F19" s="6" t="inlineStr">
         <is>
           <t>expected → 20E</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>alongside · 20E</t>
         </is>
       </c>
     </row>
@@ -962,6 +1004,11 @@
           <t>expected → 20AB</t>
         </is>
       </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>expected · 20AB (marked, P.B slipped to 04/15)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -982,6 +1029,11 @@
           <t>expected → 20B</t>
         </is>
       </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20B (P.B slipped to 04/10)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -1000,6 +1052,11 @@
       <c r="F22" s="6" t="inlineStr">
         <is>
           <t>expected → 20AB</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>alongside · 20AB (ETD now 04/17)</t>
         </is>
       </c>
     </row>
@@ -1018,6 +1075,11 @@
           <t>expected · 20B (new)</t>
         </is>
       </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20AB</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -1034,6 +1096,11 @@
           <t>expected · 20C (new, first since reopening)</t>
         </is>
       </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20C</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -1050,6 +1117,11 @@
           <t>expected · 20D (new, barge)</t>
         </is>
       </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>alongside · 20D</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -1064,6 +1136,28 @@
       <c r="F26" s="5" t="inlineStr">
         <is>
           <t>expected · 20F (new)</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20F</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>SAWASDEE SPICA</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr"/>
+      <c r="C27" s="5" t="inlineStr"/>
+      <c r="D27" s="5" t="inlineStr"/>
+      <c r="E27" s="5" t="inlineStr"/>
+      <c r="F27" s="5" t="inlineStr"/>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20B (new)</t>
         </is>
       </c>
     </row>
@@ -1108,7 +1202,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Period (as of 02 Oct sheet)</t>
+          <t>Period (as of 03 Oct sheet)</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -3356,4 +3450,427 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PAT Berth Window — Vessel List by Berth — Sheet dated 03 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Berth</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Vessel</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>LOA (m)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>ETA</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>P.B</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>ETD</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Hours Alongside</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Shift</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Marked</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>RESURGENCE</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="n">
+        <v>458</v>
+      </c>
+      <c r="D4" s="8" t="n">
+        <v>46298.5</v>
+      </c>
+      <c r="E4" s="8" t="n">
+        <v>46298.5</v>
+      </c>
+      <c r="F4" s="8" t="n">
+        <v>46299.70833333334</v>
+      </c>
+      <c r="G4" s="9">
+        <f>(F4-E4)*24</f>
+        <v/>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I4" s="7" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>ZHONG GU BEI HAI</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="n">
+        <v>561</v>
+      </c>
+      <c r="D5" s="11" t="n">
+        <v>46299.375</v>
+      </c>
+      <c r="E5" s="11" t="n">
+        <v>46299.625</v>
+      </c>
+      <c r="F5" s="11" t="n">
+        <v>46301.41666666666</v>
+      </c>
+      <c r="G5" s="12">
+        <f>(F5-E5)*24</f>
+        <v/>
+      </c>
+      <c r="H5" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I5" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>JOSCO LUCKY</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>564</v>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>46300.91666666666</v>
+      </c>
+      <c r="E6" s="8" t="n">
+        <v>46301.5</v>
+      </c>
+      <c r="F6" s="8" t="n">
+        <v>46302.54166666666</v>
+      </c>
+      <c r="G6" s="9">
+        <f>(F6-E6)*24</f>
+        <v/>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I6" s="7" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>YM IMPROVEMENT</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>564</v>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>46298.95833333334</v>
+      </c>
+      <c r="E7" s="8" t="n">
+        <v>46299.41666666666</v>
+      </c>
+      <c r="F7" s="8" t="n">
+        <v>46300.5</v>
+      </c>
+      <c r="G7" s="9">
+        <f>(F7-E7)*24</f>
+        <v/>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>SAWASDEE SPICA</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>564</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>46300.83333333334</v>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>46300.83333333334</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>46302.5</v>
+      </c>
+      <c r="G8" s="9">
+        <f>(F8-E8)*24</f>
+        <v/>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I8" s="7" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>SAWASDEE DENEB</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>564</v>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E9" s="8" t="n">
+        <v>46300.5</v>
+      </c>
+      <c r="F9" s="8" t="n">
+        <v>46302.5</v>
+      </c>
+      <c r="G9" s="9">
+        <f>(F9-E9)*24</f>
+        <v/>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I9" s="7" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>HARI BHUM (Barge)</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>259</v>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>46298.20833333334</v>
+      </c>
+      <c r="E10" s="8" t="n">
+        <v>46298.20833333334</v>
+      </c>
+      <c r="F10" s="8" t="n">
+        <v>46298.66666666666</v>
+      </c>
+      <c r="G10" s="9">
+        <f>(F10-E10)*24</f>
+        <v/>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I10" s="7" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>20E</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>WAN HAI 278</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>564</v>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>46297.75</v>
+      </c>
+      <c r="E11" s="8" t="n">
+        <v>46298.41666666666</v>
+      </c>
+      <c r="F11" s="8" t="n">
+        <v>46300.45833333334</v>
+      </c>
+      <c r="G11" s="9">
+        <f>(F11-E11)*24</f>
+        <v/>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>KMTC BANGKOK</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>565</v>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>46297.29166666666</v>
+      </c>
+      <c r="E12" s="8" t="n">
+        <v>46297.33333333334</v>
+      </c>
+      <c r="F12" s="8" t="n">
+        <v>46298.70833333334</v>
+      </c>
+      <c r="G12" s="9">
+        <f>(F12-E12)*24</f>
+        <v/>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I12" s="7" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>XIN MING ZHOU 98</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>564</v>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>46299.375</v>
+      </c>
+      <c r="E13" s="8" t="n">
+        <v>46299.375</v>
+      </c>
+      <c r="F13" s="8" t="n">
+        <v>46300.375</v>
+      </c>
+      <c r="G13" s="9">
+        <f>(F13-E13)*24</f>
+        <v/>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I13" s="7" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update 03 Oct 2026 from berthing-section sheet: ETA/P.B/ETD, new notices, 20D closure to 25 Oct
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01-10-2026/PAT_Berth_Window.xlsx
+++ b/01-10-2026/PAT_Berth_Window.xlsx
@@ -952,7 +952,7 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>alongside · 20F</t>
+          <t>alongside · 20F (D&amp;T 02/11)</t>
         </is>
       </c>
     </row>
@@ -981,7 +981,7 @@
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>alongside · 20E</t>
+          <t>at anchorage · 20E (ETA 02/22, P.B 03/10)</t>
         </is>
       </c>
     </row>
@@ -1056,7 +1056,7 @@
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>alongside · 20AB (ETD now 04/17)</t>
+          <t>expected · 20AB (ETD now 04/17)</t>
         </is>
       </c>
     </row>
@@ -1077,7 +1077,7 @@
       </c>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>expected → 20AB</t>
+          <t>expected → 20B</t>
         </is>
       </c>
     </row>
@@ -1119,7 +1119,7 @@
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>alongside · 20D</t>
+          <t>alongside · 20D (D&amp;T 03/07)</t>
         </is>
       </c>
     </row>
@@ -1157,7 +1157,7 @@
       <c r="F27" s="5" t="inlineStr"/>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>expected · 20B (new)</t>
+          <t>feeder sheet only · 20B (not on berthing sheet)</t>
         </is>
       </c>
     </row>
@@ -1256,7 +1256,7 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Closed until 5 Oct 2026 (slipped 1→3→5 Oct)</t>
+          <t>Closed until 5 Oct 2026 (slipped 1→3→5 Oct); cable splicing 4 Oct 09:00–12:00</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>4–24 Oct 2026 (slipped 1–21→3–24→4–24 Oct)</t>
+          <t>4–25 Oct 2026 (end date moved 24→25 on 03 Oct berthing sheet)</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -1293,7 +1293,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Berth closed 4–24 Oct 2026 to renovate electric channel</t>
+          <t>Berth closed 4–25 Oct 2026 to renovate electric channel</t>
         </is>
       </c>
     </row>
@@ -1310,7 +1310,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>5–18 Oct 2026 (slipped 1–15→3–18→5–18 Oct)</t>
+          <t>From 5 Oct 12:00 to 18 Oct 2026 (slipped 1–15→3–18→5–18 Oct)</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
@@ -3458,7 +3458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3601,25 +3601,25 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>20AB</t>
+          <t>20B</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>JOSCO LUCKY</t>
+          <t>YM IMPROVEMENT</t>
         </is>
       </c>
       <c r="C6" s="7" t="n">
         <v>564</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>46300.91666666666</v>
+        <v>46298.95833333334</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>46301.5</v>
+        <v>46299.41666666666</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>46302.54166666666</v>
+        <v>46300.5</v>
       </c>
       <c r="G6" s="9">
         <f>(F6-E6)*24</f>
@@ -3640,20 +3640,20 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>YM IMPROVEMENT</t>
+          <t>JOSCO LUCKY</t>
         </is>
       </c>
       <c r="C7" s="7" t="n">
         <v>564</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>46298.95833333334</v>
+        <v>46300.91666666666</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>46299.41666666666</v>
+        <v>46301.5</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>46300.5</v>
+        <v>46302.54166666666</v>
       </c>
       <c r="G7" s="9">
         <f>(F7-E7)*24</f>
@@ -3669,22 +3669,22 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>20B</t>
+          <t>20C</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>SAWASDEE SPICA</t>
+          <t>SAWASDEE DENEB</t>
         </is>
       </c>
       <c r="C8" s="7" t="n">
         <v>564</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>46300.83333333334</v>
+        <v>46300</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>46300.83333333334</v>
+        <v>46300.5</v>
       </c>
       <c r="F8" s="8" t="n">
         <v>46302.5</v>
@@ -3703,25 +3703,25 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>20C</t>
+          <t>20D</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>SAWASDEE DENEB</t>
+          <t>HARI BHUM (Barge)</t>
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>564</v>
+        <v>259</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>46300</v>
+        <v>46298.20833333334</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>46300.5</v>
+        <v>46298.29166666666</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>46302.5</v>
+        <v>46298.66666666666</v>
       </c>
       <c r="G9" s="9">
         <f>(F9-E9)*24</f>
@@ -3737,25 +3737,25 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>20D</t>
+          <t>20E</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>HARI BHUM (Barge)</t>
+          <t>WAN HAI 278</t>
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>259</v>
+        <v>564</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>46298.20833333334</v>
+        <v>46297.91666666666</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>46298.20833333334</v>
+        <v>46298.41666666666</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>46298.66666666666</v>
+        <v>46300.45833333334</v>
       </c>
       <c r="G10" s="9">
         <f>(F10-E10)*24</f>
@@ -3771,25 +3771,25 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>20E</t>
+          <t>20F</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>WAN HAI 278</t>
+          <t>KMTC BANGKOK</t>
         </is>
       </c>
       <c r="C11" s="7" t="n">
         <v>564</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>46297.75</v>
+        <v>46297.29166666666</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>46298.41666666666</v>
+        <v>46297.45833333334</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>46300.45833333334</v>
+        <v>46298.70833333334</v>
       </c>
       <c r="G11" s="9">
         <f>(F11-E11)*24</f>
@@ -3810,20 +3810,20 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>KMTC BANGKOK</t>
+          <t>XIN MING ZHOU 98</t>
         </is>
       </c>
       <c r="C12" s="7" t="n">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>46297.29166666666</v>
+        <v>46299.375</v>
       </c>
       <c r="E12" s="8" t="n">
-        <v>46297.33333333334</v>
+        <v>46299.375</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>46298.70833333334</v>
+        <v>46300.375</v>
       </c>
       <c r="G12" s="9">
         <f>(F12-E12)*24</f>
@@ -3835,40 +3835,6 @@
         </is>
       </c>
       <c r="I12" s="7" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>20F</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>XIN MING ZHOU 98</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="n">
-        <v>564</v>
-      </c>
-      <c r="D13" s="8" t="n">
-        <v>46299.375</v>
-      </c>
-      <c r="E13" s="8" t="n">
-        <v>46299.375</v>
-      </c>
-      <c r="F13" s="8" t="n">
-        <v>46300.375</v>
-      </c>
-      <c r="G13" s="9">
-        <f>(F13-E13)*24</f>
-        <v/>
-      </c>
-      <c r="H13" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I13" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 04 Oct 2026 ship movement data, Excel summary and history continuity
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01-10-2026/PAT_Berth_Window.xlsx
+++ b/01-10-2026/PAT_Berth_Window.xlsx
@@ -15,6 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 Oct 2026" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 Oct 2026" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 Oct 2026" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 Oct 2026" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -507,7 +508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -517,6 +518,7 @@
     <col width="36" customWidth="1" min="5" max="5"/>
     <col width="36" customWidth="1" min="6" max="6"/>
     <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -569,6 +571,11 @@
           <t>03 Oct 2026</t>
         </is>
       </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>04 Oct 2026</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -594,6 +601,7 @@
       <c r="E5" s="5" t="inlineStr"/>
       <c r="F5" s="5" t="inlineStr"/>
       <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -623,6 +631,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr"/>
       <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -644,6 +653,7 @@
       <c r="E7" s="5" t="inlineStr"/>
       <c r="F7" s="5" t="inlineStr"/>
       <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -669,6 +679,7 @@
       <c r="E8" s="5" t="inlineStr"/>
       <c r="F8" s="5" t="inlineStr"/>
       <c r="G8" s="5" t="inlineStr"/>
+      <c r="H8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -694,6 +705,7 @@
       <c r="E9" s="5" t="inlineStr"/>
       <c r="F9" s="5" t="inlineStr"/>
       <c r="G9" s="5" t="inlineStr"/>
+      <c r="H9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -715,6 +727,7 @@
       <c r="E10" s="5" t="inlineStr"/>
       <c r="F10" s="5" t="inlineStr"/>
       <c r="G10" s="5" t="inlineStr"/>
+      <c r="H10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -744,6 +757,7 @@
       </c>
       <c r="F11" s="5" t="inlineStr"/>
       <c r="G11" s="5" t="inlineStr"/>
+      <c r="H11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -765,6 +779,7 @@
       <c r="E12" s="5" t="inlineStr"/>
       <c r="F12" s="5" t="inlineStr"/>
       <c r="G12" s="5" t="inlineStr"/>
+      <c r="H12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -794,6 +809,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr"/>
       <c r="G13" s="5" t="inlineStr"/>
+      <c r="H13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -831,6 +847,7 @@
           <t>sailed (02/15)</t>
         </is>
       </c>
+      <c r="H14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -860,6 +877,7 @@
       </c>
       <c r="F15" s="5" t="inlineStr"/>
       <c r="G15" s="5" t="inlineStr"/>
+      <c r="H15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -893,6 +911,7 @@
           <t>sailed (02/17)</t>
         </is>
       </c>
+      <c r="H16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -926,6 +945,7 @@
           <t>sailed (02/17)</t>
         </is>
       </c>
+      <c r="H17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -955,6 +975,11 @@
           <t>alongside · 20F (D&amp;T 02/11)</t>
         </is>
       </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>sailed (03/17)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -982,6 +1007,11 @@
       <c r="G19" s="5" t="inlineStr">
         <is>
           <t>at anchorage · 20E (ETA 02/22, P.B 03/10)</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>alongside · 20E (P.B 03/10)</t>
         </is>
       </c>
     </row>
@@ -1009,6 +1039,11 @@
           <t>expected · 20AB (marked, P.B slipped to 04/15)</t>
         </is>
       </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>at anchorage · 20AB (ETA 04/09, P.B 04/15)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -1034,6 +1069,11 @@
           <t>expected · 20B (P.B slipped to 04/10)</t>
         </is>
       </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>alongside · 20B (P.B 04/10)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -1057,6 +1097,11 @@
       <c r="G22" s="5" t="inlineStr">
         <is>
           <t>expected · 20AB (ETD now 04/17)</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>alongside · 20AB (ETD 04/17)</t>
         </is>
       </c>
     </row>
@@ -1080,6 +1125,11 @@
           <t>expected → 20B</t>
         </is>
       </c>
+      <c r="H23" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20AB</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -1101,6 +1151,11 @@
           <t>expected · 20C</t>
         </is>
       </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20C</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -1122,6 +1177,11 @@
           <t>alongside · 20D (D&amp;T 03/07)</t>
         </is>
       </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>sailed (03/16)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -1141,6 +1201,11 @@
       <c r="G26" s="5" t="inlineStr">
         <is>
           <t>expected · 20F</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>alongside · 20F (P.B 04/09)</t>
         </is>
       </c>
     </row>
@@ -1158,6 +1223,29 @@
       <c r="G27" s="5" t="inlineStr">
         <is>
           <t>feeder sheet only · 20B (not on berthing sheet)</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20B (P.B 06/13, ETD 08/13)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>KMTC TOKYO</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr"/>
+      <c r="C28" s="5" t="inlineStr"/>
+      <c r="D28" s="5" t="inlineStr"/>
+      <c r="E28" s="5" t="inlineStr"/>
+      <c r="F28" s="5" t="inlineStr"/>
+      <c r="G28" s="5" t="inlineStr"/>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20F (new)</t>
         </is>
       </c>
     </row>
@@ -1202,7 +1290,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Period (as of 03 Oct sheet)</t>
+          <t>Period (as of 04 Oct sheet)</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -1283,7 +1371,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>4–25 Oct 2026 (end date moved 24→25 on 03 Oct berthing sheet)</t>
+          <t>4–24 Oct 2026 (03 Oct berthing sheet said 4–25)</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -1293,7 +1381,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Berth closed 4–25 Oct 2026 to renovate electric channel</t>
+          <t>Berth closed 4–24 Oct 2026 to renovate electric channel</t>
         </is>
       </c>
     </row>
@@ -3839,4 +3927,389 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PAT Berth Window — Vessel List by Berth — Sheet dated 04 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Berth</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Vessel</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>LOA (m)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>ETA</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>P.B</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>ETD</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Hours Alongside</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Shift</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Marked</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>RESURGENCE</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="n">
+        <v>458</v>
+      </c>
+      <c r="D4" s="8" t="n">
+        <v>46298.5</v>
+      </c>
+      <c r="E4" s="8" t="n">
+        <v>46298.5</v>
+      </c>
+      <c r="F4" s="8" t="n">
+        <v>46299.70833333334</v>
+      </c>
+      <c r="G4" s="9">
+        <f>(F4-E4)*24</f>
+        <v/>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I4" s="7" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>ZHONG GU BEI HAI</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>561</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>46299.375</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>46299.625</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>46301.41666666666</v>
+      </c>
+      <c r="G5" s="9">
+        <f>(F5-E5)*24</f>
+        <v/>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>JOSCO LUCKY</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>564</v>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>46300.91666666666</v>
+      </c>
+      <c r="E6" s="8" t="n">
+        <v>46301.5</v>
+      </c>
+      <c r="F6" s="8" t="n">
+        <v>46302.54166666666</v>
+      </c>
+      <c r="G6" s="9">
+        <f>(F6-E6)*24</f>
+        <v/>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I6" s="7" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>YM IMPROVEMENT</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>564</v>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>46298.95833333334</v>
+      </c>
+      <c r="E7" s="8" t="n">
+        <v>46299.41666666666</v>
+      </c>
+      <c r="F7" s="8" t="n">
+        <v>46300.5</v>
+      </c>
+      <c r="G7" s="9">
+        <f>(F7-E7)*24</f>
+        <v/>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>SAWASDEE SPICA</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>564</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>46300.875</v>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>46301.54166666666</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>46303.54166666666</v>
+      </c>
+      <c r="G8" s="9">
+        <f>(F8-E8)*24</f>
+        <v/>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I8" s="7" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>SAWASDEE DENEB</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>564</v>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E9" s="8" t="n">
+        <v>46300.5</v>
+      </c>
+      <c r="F9" s="8" t="n">
+        <v>46302.5</v>
+      </c>
+      <c r="G9" s="9">
+        <f>(F9-E9)*24</f>
+        <v/>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I9" s="7" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>20E</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>WAN HAI 278</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>564</v>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>46297.75</v>
+      </c>
+      <c r="E10" s="8" t="n">
+        <v>46298.41666666666</v>
+      </c>
+      <c r="F10" s="8" t="n">
+        <v>46300.45833333334</v>
+      </c>
+      <c r="G10" s="9">
+        <f>(F10-E10)*24</f>
+        <v/>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I10" s="7" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>XIN MING ZHOU 98</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>564</v>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>46299.375</v>
+      </c>
+      <c r="E11" s="8" t="n">
+        <v>46299.375</v>
+      </c>
+      <c r="F11" s="8" t="n">
+        <v>46300.375</v>
+      </c>
+      <c r="G11" s="9">
+        <f>(F11-E11)*24</f>
+        <v/>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>KMTC TOKYO</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>565</v>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>46301.58333333334</v>
+      </c>
+      <c r="E12" s="8" t="n">
+        <v>46301.58333333334</v>
+      </c>
+      <c r="F12" s="8" t="n">
+        <v>46303.5</v>
+      </c>
+      <c r="G12" s="9">
+        <f>(F12-E12)*24</f>
+        <v/>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I12" s="7" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add 05 Oct 2026 ship movement data, widen timeline to 11 Oct, update Excel and history
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01-10-2026/PAT_Berth_Window.xlsx
+++ b/01-10-2026/PAT_Berth_Window.xlsx
@@ -16,6 +16,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 Oct 2026" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 Oct 2026" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 Oct 2026" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 Oct 2026" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -508,7 +509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -519,6 +520,7 @@
     <col width="36" customWidth="1" min="6" max="6"/>
     <col width="40" customWidth="1" min="7" max="7"/>
     <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="42" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -576,6 +578,11 @@
           <t>04 Oct 2026</t>
         </is>
       </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>05 Oct 2026</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -602,6 +609,7 @@
       <c r="F5" s="5" t="inlineStr"/>
       <c r="G5" s="5" t="inlineStr"/>
       <c r="H5" s="5" t="inlineStr"/>
+      <c r="I5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -632,6 +640,7 @@
       <c r="F6" s="5" t="inlineStr"/>
       <c r="G6" s="5" t="inlineStr"/>
       <c r="H6" s="5" t="inlineStr"/>
+      <c r="I6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -654,6 +663,7 @@
       <c r="F7" s="5" t="inlineStr"/>
       <c r="G7" s="5" t="inlineStr"/>
       <c r="H7" s="5" t="inlineStr"/>
+      <c r="I7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -680,6 +690,7 @@
       <c r="F8" s="5" t="inlineStr"/>
       <c r="G8" s="5" t="inlineStr"/>
       <c r="H8" s="5" t="inlineStr"/>
+      <c r="I8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -706,6 +717,7 @@
       <c r="F9" s="5" t="inlineStr"/>
       <c r="G9" s="5" t="inlineStr"/>
       <c r="H9" s="5" t="inlineStr"/>
+      <c r="I9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -728,6 +740,7 @@
       <c r="F10" s="5" t="inlineStr"/>
       <c r="G10" s="5" t="inlineStr"/>
       <c r="H10" s="5" t="inlineStr"/>
+      <c r="I10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -758,6 +771,7 @@
       <c r="F11" s="5" t="inlineStr"/>
       <c r="G11" s="5" t="inlineStr"/>
       <c r="H11" s="5" t="inlineStr"/>
+      <c r="I11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -780,6 +794,7 @@
       <c r="F12" s="5" t="inlineStr"/>
       <c r="G12" s="5" t="inlineStr"/>
       <c r="H12" s="5" t="inlineStr"/>
+      <c r="I12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -810,6 +825,7 @@
       <c r="F13" s="5" t="inlineStr"/>
       <c r="G13" s="5" t="inlineStr"/>
       <c r="H13" s="5" t="inlineStr"/>
+      <c r="I13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -848,6 +864,7 @@
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr"/>
+      <c r="I14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -878,6 +895,7 @@
       <c r="F15" s="5" t="inlineStr"/>
       <c r="G15" s="5" t="inlineStr"/>
       <c r="H15" s="5" t="inlineStr"/>
+      <c r="I15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -912,6 +930,7 @@
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr"/>
+      <c r="I16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -946,6 +965,7 @@
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr"/>
+      <c r="I17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -980,6 +1000,7 @@
           <t>sailed (03/17)</t>
         </is>
       </c>
+      <c r="I18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -1012,6 +1033,11 @@
       <c r="H19" s="5" t="inlineStr">
         <is>
           <t>alongside · 20E (P.B 03/10)</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>alongside · 20E (ETD 05/11)</t>
         </is>
       </c>
     </row>
@@ -1044,6 +1070,11 @@
           <t>at anchorage · 20AB (ETA 04/09, P.B 04/15)</t>
         </is>
       </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>alongside · 20AB (ETD slipped to 06/11)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -1074,6 +1105,11 @@
           <t>alongside · 20B (P.B 04/10)</t>
         </is>
       </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>alongside · 20B (ETD 05/12)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -1102,6 +1138,11 @@
       <c r="H22" s="5" t="inlineStr">
         <is>
           <t>alongside · 20AB (ETD 04/17)</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>sailed (04/17)</t>
         </is>
       </c>
     </row>
@@ -1130,6 +1171,11 @@
           <t>expected → 20AB</t>
         </is>
       </c>
+      <c r="I23" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20D (P.B 06/18)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -1156,6 +1202,11 @@
           <t>expected · 20C</t>
         </is>
       </c>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>at anchorage · 20C (P.B 05/12)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -1182,6 +1233,7 @@
           <t>sailed (03/16)</t>
         </is>
       </c>
+      <c r="I25" s="5" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -1206,6 +1258,11 @@
       <c r="H26" s="5" t="inlineStr">
         <is>
           <t>alongside · 20F (P.B 04/09)</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>sailed (05/09)</t>
         </is>
       </c>
     </row>
@@ -1228,6 +1285,11 @@
       <c r="H27" s="5" t="inlineStr">
         <is>
           <t>expected · 20B (P.B 06/13, ETD 08/13)</t>
+        </is>
+      </c>
+      <c r="I27" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20B</t>
         </is>
       </c>
     </row>
@@ -1246,6 +1308,552 @@
       <c r="H28" s="5" t="inlineStr">
         <is>
           <t>expected · 20F (new)</t>
+        </is>
+      </c>
+      <c r="I28" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20AB (ETA 06/13)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>GREEN PARK</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr"/>
+      <c r="C29" s="5" t="inlineStr"/>
+      <c r="D29" s="5" t="inlineStr"/>
+      <c r="E29" s="5" t="inlineStr"/>
+      <c r="F29" s="5" t="inlineStr"/>
+      <c r="G29" s="5" t="inlineStr"/>
+      <c r="H29" s="5" t="inlineStr"/>
+      <c r="I29" s="6" t="inlineStr">
+        <is>
+          <t>expected · 20AB (new, marked)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>SAWASDEE ATLANTIC</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr"/>
+      <c r="C30" s="5" t="inlineStr"/>
+      <c r="D30" s="5" t="inlineStr"/>
+      <c r="E30" s="5" t="inlineStr"/>
+      <c r="F30" s="5" t="inlineStr"/>
+      <c r="G30" s="5" t="inlineStr"/>
+      <c r="H30" s="5" t="inlineStr"/>
+      <c r="I30" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20C (new)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>MTT BANGKOK</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr"/>
+      <c r="C31" s="5" t="inlineStr"/>
+      <c r="D31" s="5" t="inlineStr"/>
+      <c r="E31" s="5" t="inlineStr"/>
+      <c r="F31" s="5" t="inlineStr"/>
+      <c r="G31" s="5" t="inlineStr"/>
+      <c r="H31" s="5" t="inlineStr"/>
+      <c r="I31" s="6" t="inlineStr">
+        <is>
+          <t>expected · 20D (new, marked)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>XIN AN</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr"/>
+      <c r="C32" s="5" t="inlineStr"/>
+      <c r="D32" s="5" t="inlineStr"/>
+      <c r="E32" s="5" t="inlineStr"/>
+      <c r="F32" s="5" t="inlineStr"/>
+      <c r="G32" s="5" t="inlineStr"/>
+      <c r="H32" s="5" t="inlineStr"/>
+      <c r="I32" s="6" t="inlineStr">
+        <is>
+          <t>expected · 20F (new, marked)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PAT Berth Window — Vessel List by Berth — Sheet dated 05 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Berth</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Vessel</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>LOA (m)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>ETA</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>P.B</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>ETD</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Hours Alongside</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Shift</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Marked</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>ZHONG GU BEI HAI</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="n">
+        <v>561</v>
+      </c>
+      <c r="D4" s="8" t="n">
+        <v>46299.375</v>
+      </c>
+      <c r="E4" s="8" t="n">
+        <v>46299.625</v>
+      </c>
+      <c r="F4" s="8" t="n">
+        <v>46301.45833333334</v>
+      </c>
+      <c r="G4" s="9">
+        <f>(F4-E4)*24</f>
+        <v/>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I4" s="7" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>KMTC TOKYO</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>565</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>46301.54166666666</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>46301.54166666666</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>46303.5</v>
+      </c>
+      <c r="G5" s="9">
+        <f>(F5-E5)*24</f>
+        <v/>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>GREEN PARK</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="n">
+        <v>482</v>
+      </c>
+      <c r="D6" s="11" t="n">
+        <v>46302.45833333334</v>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>46303.625</v>
+      </c>
+      <c r="F6" s="11" t="n">
+        <v>46304.58333333334</v>
+      </c>
+      <c r="G6" s="12">
+        <f>(F6-E6)*24</f>
+        <v/>
+      </c>
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I6" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>YM IMPROVEMENT</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>564</v>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>46298.95833333334</v>
+      </c>
+      <c r="E7" s="8" t="n">
+        <v>46299.41666666666</v>
+      </c>
+      <c r="F7" s="8" t="n">
+        <v>46300.5</v>
+      </c>
+      <c r="G7" s="9">
+        <f>(F7-E7)*24</f>
+        <v/>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>SAWASDEE SPICA</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>564</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>46300.875</v>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>46301.54166666666</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>46303.54166666666</v>
+      </c>
+      <c r="G8" s="9">
+        <f>(F8-E8)*24</f>
+        <v/>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I8" s="7" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>SAWASDEE DENEB</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>564</v>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E9" s="8" t="n">
+        <v>46300.5</v>
+      </c>
+      <c r="F9" s="8" t="n">
+        <v>46302.5</v>
+      </c>
+      <c r="G9" s="9">
+        <f>(F9-E9)*24</f>
+        <v/>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I9" s="7" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>SAWASDEE ATLANTIC</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>564</v>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>46302.91666666666</v>
+      </c>
+      <c r="E10" s="8" t="n">
+        <v>46303.625</v>
+      </c>
+      <c r="F10" s="8" t="n">
+        <v>46305.54166666666</v>
+      </c>
+      <c r="G10" s="9">
+        <f>(F10-E10)*24</f>
+        <v/>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I10" s="7" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>JOSCO LUCKY</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>564</v>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>46301.75</v>
+      </c>
+      <c r="E11" s="8" t="n">
+        <v>46301.75</v>
+      </c>
+      <c r="F11" s="8" t="n">
+        <v>46302.625</v>
+      </c>
+      <c r="G11" s="9">
+        <f>(F11-E11)*24</f>
+        <v/>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>MTT BANGKOK</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="n">
+        <v>564</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>46302.625</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>46302.70833333334</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>46304.54166666666</v>
+      </c>
+      <c r="G12" s="12">
+        <f>(F12-E12)*24</f>
+        <v/>
+      </c>
+      <c r="H12" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I12" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>20E</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>WAN HAI 278</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>564</v>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>46297.75</v>
+      </c>
+      <c r="E13" s="8" t="n">
+        <v>46298.41666666666</v>
+      </c>
+      <c r="F13" s="8" t="n">
+        <v>46300.45833333334</v>
+      </c>
+      <c r="G13" s="9">
+        <f>(F13-E13)*24</f>
+        <v/>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I13" s="7" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>XIN AN</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="n">
+        <v>564</v>
+      </c>
+      <c r="D14" s="11" t="n">
+        <v>46302.58333333334</v>
+      </c>
+      <c r="E14" s="11" t="n">
+        <v>46302.70833333334</v>
+      </c>
+      <c r="F14" s="11" t="n">
+        <v>46304.54166666666</v>
+      </c>
+      <c r="G14" s="12">
+        <f>(F14-E14)*24</f>
+        <v/>
+      </c>
+      <c r="H14" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I14" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1290,7 +1898,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Period (as of 04 Oct sheet)</t>
+          <t>Period (as of 05 Oct sheet)</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -1344,7 +1952,7 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Closed until 5 Oct 2026 (slipped 1→3→5 Oct); cable splicing 4 Oct 09:00–12:00</t>
+          <t>Closed until 5 Oct 2026 (slipped 1→3→5 Oct); reopened – no notice on the 05 Oct sheet</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -1371,7 +1979,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>4–24 Oct 2026 (03 Oct berthing sheet said 4–25)</t>
+          <t>4–24 Oct 2026 (but JOSCO LUCKY / MTT BANGKOK are booked from 06/18 – please confirm)</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Excel: Berth Notices sheet now logs every day's notices with change tracking
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01-10-2026/PAT_Berth_Window.xlsx
+++ b/01-10-2026/PAT_Berth_Window.xlsx
@@ -18,17 +18,20 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 Oct 2026" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 Oct 2026" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Berth Notices'!$A$4:$G$32</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="dd-mmm hh:mm"/>
-    <numFmt numFmtId="166" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="dd-mmm-yyyy"/>
+    <numFmt numFmtId="166" formatCode="dd-mmm hh:mm"/>
+    <numFmt numFmtId="167" formatCode="0.0"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -84,7 +87,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -106,11 +109,25 @@
         <color rgb="00D9D9D9"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="medium">
+        <color rgb="0016324F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -126,8 +143,14 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -135,13 +158,52 @@
     <xf numFmtId="166" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="166" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1482,28 +1544,28 @@
           <t>ZHONG GU BEI HAI</t>
         </is>
       </c>
-      <c r="C4" s="7" t="n">
+      <c r="C4" s="23" t="n">
         <v>561</v>
       </c>
-      <c r="D4" s="8" t="n">
+      <c r="D4" s="11" t="n">
         <v>46299.375</v>
       </c>
-      <c r="E4" s="8" t="n">
+      <c r="E4" s="11" t="n">
         <v>46299.625</v>
       </c>
-      <c r="F4" s="8" t="n">
+      <c r="F4" s="11" t="n">
         <v>46301.45833333334</v>
       </c>
-      <c r="G4" s="9">
+      <c r="G4" s="26">
         <f>(F4-E4)*24</f>
         <v/>
       </c>
-      <c r="H4" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I4" s="7" t="inlineStr"/>
+      <c r="H4" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I4" s="23" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -1516,28 +1578,28 @@
           <t>KMTC TOKYO</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C5" s="23" t="n">
         <v>565</v>
       </c>
-      <c r="D5" s="8" t="n">
+      <c r="D5" s="11" t="n">
         <v>46301.54166666666</v>
       </c>
-      <c r="E5" s="8" t="n">
+      <c r="E5" s="11" t="n">
         <v>46301.54166666666</v>
       </c>
-      <c r="F5" s="8" t="n">
+      <c r="F5" s="11" t="n">
         <v>46303.5</v>
       </c>
-      <c r="G5" s="9">
+      <c r="G5" s="26">
         <f>(F5-E5)*24</f>
         <v/>
       </c>
-      <c r="H5" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I5" s="7" t="inlineStr"/>
+      <c r="H5" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I5" s="23" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -1550,28 +1612,28 @@
           <t>GREEN PARK</t>
         </is>
       </c>
-      <c r="C6" s="10" t="n">
+      <c r="C6" s="17" t="n">
         <v>482</v>
       </c>
-      <c r="D6" s="11" t="n">
+      <c r="D6" s="25" t="n">
         <v>46302.45833333334</v>
       </c>
-      <c r="E6" s="11" t="n">
+      <c r="E6" s="25" t="n">
         <v>46303.625</v>
       </c>
-      <c r="F6" s="11" t="n">
+      <c r="F6" s="25" t="n">
         <v>46304.58333333334</v>
       </c>
-      <c r="G6" s="12">
+      <c r="G6" s="27">
         <f>(F6-E6)*24</f>
         <v/>
       </c>
-      <c r="H6" s="10" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I6" s="10" t="inlineStr">
+      <c r="H6" s="17" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I6" s="17" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -1588,28 +1650,28 @@
           <t>YM IMPROVEMENT</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C7" s="23" t="n">
         <v>564</v>
       </c>
-      <c r="D7" s="8" t="n">
+      <c r="D7" s="11" t="n">
         <v>46298.95833333334</v>
       </c>
-      <c r="E7" s="8" t="n">
+      <c r="E7" s="11" t="n">
         <v>46299.41666666666</v>
       </c>
-      <c r="F7" s="8" t="n">
+      <c r="F7" s="11" t="n">
         <v>46300.5</v>
       </c>
-      <c r="G7" s="9">
+      <c r="G7" s="26">
         <f>(F7-E7)*24</f>
         <v/>
       </c>
-      <c r="H7" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I7" s="7" t="inlineStr"/>
+      <c r="H7" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I7" s="23" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -1622,28 +1684,28 @@
           <t>SAWASDEE SPICA</t>
         </is>
       </c>
-      <c r="C8" s="7" t="n">
+      <c r="C8" s="23" t="n">
         <v>564</v>
       </c>
-      <c r="D8" s="8" t="n">
+      <c r="D8" s="11" t="n">
         <v>46300.875</v>
       </c>
-      <c r="E8" s="8" t="n">
+      <c r="E8" s="11" t="n">
         <v>46301.54166666666</v>
       </c>
-      <c r="F8" s="8" t="n">
+      <c r="F8" s="11" t="n">
         <v>46303.54166666666</v>
       </c>
-      <c r="G8" s="9">
+      <c r="G8" s="26">
         <f>(F8-E8)*24</f>
         <v/>
       </c>
-      <c r="H8" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I8" s="7" t="inlineStr"/>
+      <c r="H8" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I8" s="23" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -1656,28 +1718,28 @@
           <t>SAWASDEE DENEB</t>
         </is>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="C9" s="23" t="n">
         <v>564</v>
       </c>
-      <c r="D9" s="8" t="n">
+      <c r="D9" s="11" t="n">
         <v>46300</v>
       </c>
-      <c r="E9" s="8" t="n">
+      <c r="E9" s="11" t="n">
         <v>46300.5</v>
       </c>
-      <c r="F9" s="8" t="n">
+      <c r="F9" s="11" t="n">
         <v>46302.5</v>
       </c>
-      <c r="G9" s="9">
+      <c r="G9" s="26">
         <f>(F9-E9)*24</f>
         <v/>
       </c>
-      <c r="H9" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I9" s="7" t="inlineStr"/>
+      <c r="H9" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I9" s="23" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -1690,28 +1752,28 @@
           <t>SAWASDEE ATLANTIC</t>
         </is>
       </c>
-      <c r="C10" s="7" t="n">
+      <c r="C10" s="23" t="n">
         <v>564</v>
       </c>
-      <c r="D10" s="8" t="n">
+      <c r="D10" s="11" t="n">
         <v>46302.91666666666</v>
       </c>
-      <c r="E10" s="8" t="n">
+      <c r="E10" s="11" t="n">
         <v>46303.625</v>
       </c>
-      <c r="F10" s="8" t="n">
+      <c r="F10" s="11" t="n">
         <v>46305.54166666666</v>
       </c>
-      <c r="G10" s="9">
+      <c r="G10" s="26">
         <f>(F10-E10)*24</f>
         <v/>
       </c>
-      <c r="H10" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I10" s="7" t="inlineStr"/>
+      <c r="H10" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I10" s="23" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -1724,28 +1786,28 @@
           <t>JOSCO LUCKY</t>
         </is>
       </c>
-      <c r="C11" s="7" t="n">
+      <c r="C11" s="23" t="n">
         <v>564</v>
       </c>
-      <c r="D11" s="8" t="n">
+      <c r="D11" s="11" t="n">
         <v>46301.75</v>
       </c>
-      <c r="E11" s="8" t="n">
+      <c r="E11" s="11" t="n">
         <v>46301.75</v>
       </c>
-      <c r="F11" s="8" t="n">
+      <c r="F11" s="11" t="n">
         <v>46302.625</v>
       </c>
-      <c r="G11" s="9">
+      <c r="G11" s="26">
         <f>(F11-E11)*24</f>
         <v/>
       </c>
-      <c r="H11" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I11" s="7" t="inlineStr"/>
+      <c r="H11" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I11" s="23" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
@@ -1758,28 +1820,28 @@
           <t>MTT BANGKOK</t>
         </is>
       </c>
-      <c r="C12" s="10" t="n">
+      <c r="C12" s="17" t="n">
         <v>564</v>
       </c>
-      <c r="D12" s="11" t="n">
+      <c r="D12" s="25" t="n">
         <v>46302.625</v>
       </c>
-      <c r="E12" s="11" t="n">
+      <c r="E12" s="25" t="n">
         <v>46302.70833333334</v>
       </c>
-      <c r="F12" s="11" t="n">
+      <c r="F12" s="25" t="n">
         <v>46304.54166666666</v>
       </c>
-      <c r="G12" s="12">
+      <c r="G12" s="27">
         <f>(F12-E12)*24</f>
         <v/>
       </c>
-      <c r="H12" s="10" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I12" s="10" t="inlineStr">
+      <c r="H12" s="17" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I12" s="17" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -1796,28 +1858,28 @@
           <t>WAN HAI 278</t>
         </is>
       </c>
-      <c r="C13" s="7" t="n">
+      <c r="C13" s="23" t="n">
         <v>564</v>
       </c>
-      <c r="D13" s="8" t="n">
+      <c r="D13" s="11" t="n">
         <v>46297.75</v>
       </c>
-      <c r="E13" s="8" t="n">
+      <c r="E13" s="11" t="n">
         <v>46298.41666666666</v>
       </c>
-      <c r="F13" s="8" t="n">
+      <c r="F13" s="11" t="n">
         <v>46300.45833333334</v>
       </c>
-      <c r="G13" s="9">
+      <c r="G13" s="26">
         <f>(F13-E13)*24</f>
         <v/>
       </c>
-      <c r="H13" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I13" s="7" t="inlineStr"/>
+      <c r="H13" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I13" s="23" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
@@ -1830,28 +1892,28 @@
           <t>XIN AN</t>
         </is>
       </c>
-      <c r="C14" s="10" t="n">
+      <c r="C14" s="17" t="n">
         <v>564</v>
       </c>
-      <c r="D14" s="11" t="n">
+      <c r="D14" s="25" t="n">
         <v>46302.58333333334</v>
       </c>
-      <c r="E14" s="11" t="n">
+      <c r="E14" s="25" t="n">
         <v>46302.70833333334</v>
       </c>
-      <c r="F14" s="11" t="n">
+      <c r="F14" s="25" t="n">
         <v>46304.54166666666</v>
       </c>
-      <c r="G14" s="12">
+      <c r="G14" s="27">
         <f>(F14-E14)*24</f>
         <v/>
       </c>
-      <c r="H14" s="10" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I14" s="10" t="inlineStr">
+      <c r="H14" s="17" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I14" s="17" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -1868,159 +1930,962 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="66" customWidth="1" min="6" max="6"/>
+    <col width="52" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Berth Closures &amp; Gate Stoppages (as announced, by sheet date)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+          <t>Berth Closures &amp; Gate Stoppages — Daily Log (every sheet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>One row per notice printed on each day's sheet. From / To are inclusive dates (times shown when the sheet gives them). For 20C, ‘To’ is the date the wharf is to be utilised again. Highlighted rows = new, moved or slipped compared with the previous sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Sheet Date</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Berth / Gate</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>First Announced</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Period (as of 05 Oct sheet)</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Notice Text</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>From</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>To</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Notice (as printed, English)</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Change vs previous sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="n">
+        <v>46212</v>
+      </c>
+      <c r="E5" s="10" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>20C closed 9 Jul – 30 Sep 2026 (cable track repair)</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>First sheet in the log</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Cable splicing</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="n">
+        <v>46295.35416666666</v>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>46295.6875</v>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>20D 30 Sep 08:30–16:30 (cable splicing)</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>First sheet in the log</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>20AB / G.29</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>29 Sep sheet</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>29–30 Sep 2026 (ended)</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="C7" s="13" t="inlineStr">
         <is>
           <t>Gate stopped</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="D7" s="14" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E7" s="14" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F7" s="13" t="inlineStr">
         <is>
           <t>G.29 stops working 29–30 Sep 2026 to repair spreader</t>
         </is>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="G7" s="13" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="15" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
         <is>
           <t>20C</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>29 Sep sheet</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>Closed until 5 Oct 2026 (slipped 1→3→5 Oct); reopened – no notice on the 05 Oct sheet</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="C8" s="16" t="inlineStr">
         <is>
           <t>Berth closed</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>Wharf to be utilised from 5 Oct 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="D8" s="17" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E8" s="18" t="n">
+        <v>46296</v>
+      </c>
+      <c r="F8" s="16" t="inlineStr">
+        <is>
+          <t>Wharf will be utilised on 1 Oct 2026</t>
+        </is>
+      </c>
+      <c r="G8" s="16" t="inlineStr">
+        <is>
+          <t>Reopening moved 30 Sep → 1 Oct</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="15" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
         <is>
           <t>20D</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>29 Sep sheet</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>4–24 Oct 2026 (but JOSCO LUCKY / MTT BANGKOK are booked from 06/18 – please confirm)</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="C9" s="16" t="inlineStr">
         <is>
           <t>Berth closed</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>Berth closed 4–24 Oct 2026 to renovate electric channel</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="D9" s="18" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E9" s="18" t="n">
+        <v>46316</v>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>Close on 1–21 Oct 2026 to renovate electric channel</t>
+        </is>
+      </c>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>New (replaces the 30 Sep splicing notice)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="15" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B10" s="16" t="inlineStr">
         <is>
           <t>20E / G.25</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>29 Sep sheet</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>From 5 Oct 12:00 to 18 Oct 2026 (slipped 1–15→3–18→5–18 Oct)</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="C10" s="16" t="inlineStr">
         <is>
           <t>Gate stopped</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="D10" s="18" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E10" s="18" t="n">
+        <v>46310</v>
+      </c>
+      <c r="F10" s="16" t="inlineStr">
+        <is>
+          <t>G.25 stops working 1–15 Oct 2026 to change trolley rail</t>
+        </is>
+      </c>
+      <c r="G10" s="16" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="19" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B11" s="20" t="inlineStr">
+        <is>
+          <t>20AB / G.29</t>
+        </is>
+      </c>
+      <c r="C11" s="20" t="inlineStr">
+        <is>
+          <t>Gate stopped</t>
+        </is>
+      </c>
+      <c r="D11" s="21" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E11" s="21" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F11" s="20" t="inlineStr">
+        <is>
+          <t>G.29 stops working 29–30 Sep 2026 to repair spreader</t>
+        </is>
+      </c>
+      <c r="G11" s="20" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="15" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="D12" s="17" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E12" s="18" t="n">
+        <v>46298</v>
+      </c>
+      <c r="F12" s="16" t="inlineStr">
+        <is>
+          <t>Wharf will be utilised on 3 Oct 2026</t>
+        </is>
+      </c>
+      <c r="G12" s="16" t="inlineStr">
+        <is>
+          <t>Slipped: reopening 1 Oct → 3 Oct</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="D13" s="18" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E13" s="18" t="n">
+        <v>46319</v>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>Close on 3–24 Oct 2026 to renovate electric channel</t>
+        </is>
+      </c>
+      <c r="G13" s="16" t="inlineStr">
+        <is>
+          <t>Slipped: 1–21 Oct → 3–24 Oct</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>20E / G.25</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="inlineStr">
+        <is>
+          <t>Gate stopped</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E14" s="18" t="n">
+        <v>46313</v>
+      </c>
+      <c r="F14" s="16" t="inlineStr">
+        <is>
+          <t>G.25 stops working 3–18 Oct 2026 to change trolley rail</t>
+        </is>
+      </c>
+      <c r="G14" s="16" t="inlineStr">
+        <is>
+          <t>Slipped: 1–15 Oct → 3–18 Oct</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>20AB / G.29</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>Gate stopped</t>
+        </is>
+      </c>
+      <c r="D15" s="22" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E15" s="22" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F15" s="13" t="inlineStr">
+        <is>
+          <t>(no longer listed – 29–30 Sep period has ended)</t>
+        </is>
+      </c>
+      <c r="G15" s="13" t="inlineStr">
+        <is>
+          <t>Dropped from sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="D16" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E16" s="10" t="n">
+        <v>46298</v>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>Wharf will be utilised on 3 Oct (sheet prints 2027, treated as a typo)</t>
+        </is>
+      </c>
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E17" s="10" t="n">
+        <v>46319</v>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>Close on 3–24 Oct 2026 to renovate electric channel</t>
+        </is>
+      </c>
+      <c r="G17" s="9" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>20E / G.25</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>Gate stopped</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E18" s="10" t="n">
+        <v>46313</v>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>G.25 stops working 3–18 Oct 2026 to change trolley rail</t>
+        </is>
+      </c>
+      <c r="G18" s="9" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="C19" s="13" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="D19" s="22" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E19" s="14" t="n">
+        <v>46300</v>
+      </c>
+      <c r="F19" s="13" t="inlineStr">
+        <is>
+          <t>Wharf will be utilised on 5 Oct 2026</t>
+        </is>
+      </c>
+      <c r="G19" s="13" t="inlineStr">
+        <is>
+          <t>Slipped: reopening 3 Oct → 5 Oct</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="15" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B20" s="16" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="C20" s="16" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E20" s="18" t="n">
+        <v>46319</v>
+      </c>
+      <c r="F20" s="16" t="inlineStr">
+        <is>
+          <t>Close on 4–24 Oct 2026 to renovate electric channel</t>
+        </is>
+      </c>
+      <c r="G20" s="16" t="inlineStr">
+        <is>
+          <t>Slipped: start 3 Oct → 4 Oct</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="15" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>20E / G.25</t>
+        </is>
+      </c>
+      <c r="C21" s="16" t="inlineStr">
+        <is>
+          <t>Gate stopped</t>
+        </is>
+      </c>
+      <c r="D21" s="18" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E21" s="18" t="n">
+        <v>46313</v>
+      </c>
+      <c r="F21" s="16" t="inlineStr">
         <is>
           <t>G.25 stops working 5–18 Oct 2026 to change trolley rail</t>
         </is>
       </c>
+      <c r="G21" s="16" t="inlineStr">
+        <is>
+          <t>Slipped: start 3 Oct → 5 Oct</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="19" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B22" s="20" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="C22" s="20" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="D22" s="24" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E22" s="21" t="n">
+        <v>46300</v>
+      </c>
+      <c r="F22" s="20" t="inlineStr">
+        <is>
+          <t>Wharf will be utilised on 5 Oct 2026</t>
+        </is>
+      </c>
+      <c r="G22" s="20" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="15" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B23" s="16" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="C23" s="16" t="inlineStr">
+        <is>
+          <t>Cable splicing</t>
+        </is>
+      </c>
+      <c r="D23" s="25" t="n">
+        <v>46299.375</v>
+      </c>
+      <c r="E23" s="25" t="n">
+        <v>46299.5</v>
+      </c>
+      <c r="F23" s="16" t="inlineStr">
+        <is>
+          <t>20C and 20D cable splicing on 4 Oct 2026, 09:00–12:00</t>
+        </is>
+      </c>
+      <c r="G23" s="16" t="inlineStr">
+        <is>
+          <t>New (berthing-section sheet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="15" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B24" s="16" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="C24" s="16" t="inlineStr">
+        <is>
+          <t>Cable splicing</t>
+        </is>
+      </c>
+      <c r="D24" s="25" t="n">
+        <v>46299.375</v>
+      </c>
+      <c r="E24" s="25" t="n">
+        <v>46299.5</v>
+      </c>
+      <c r="F24" s="16" t="inlineStr">
+        <is>
+          <t>20C and 20D cable splicing on 4 Oct 2026, 09:00–12:00</t>
+        </is>
+      </c>
+      <c r="G24" s="16" t="inlineStr">
+        <is>
+          <t>New (berthing-section sheet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="15" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B25" s="16" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="C25" s="16" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="D25" s="18" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E25" s="18" t="n">
+        <v>46320</v>
+      </c>
+      <c r="F25" s="16" t="inlineStr">
+        <is>
+          <t>20D closed 4–25 Oct 2026 to renovate electric channel (cable track bays 1700–1800)</t>
+        </is>
+      </c>
+      <c r="G25" s="16" t="inlineStr">
+        <is>
+          <t>End moved 24 → 25 Oct (the feeder sheet of the same day still says 24)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="15" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B26" s="16" t="inlineStr">
+        <is>
+          <t>20E / G.25</t>
+        </is>
+      </c>
+      <c r="C26" s="16" t="inlineStr">
+        <is>
+          <t>Gate stopped</t>
+        </is>
+      </c>
+      <c r="D26" s="25" t="n">
+        <v>46300.5</v>
+      </c>
+      <c r="E26" s="18" t="n">
+        <v>46313</v>
+      </c>
+      <c r="F26" s="16" t="inlineStr">
+        <is>
+          <t>G.25 stops working from 5 Oct 12:00 to change trolley rail (bays 700–900); end date is cut off on this sheet, daily sheet says 18 Oct</t>
+        </is>
+      </c>
+      <c r="G26" s="16" t="inlineStr">
+        <is>
+          <t>Start time added (12:00); end date unclear</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="19" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B27" s="20" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="C27" s="20" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="D27" s="24" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E27" s="21" t="n">
+        <v>46300</v>
+      </c>
+      <c r="F27" s="20" t="inlineStr">
+        <is>
+          <t>Wharf will be utilised on 5 Oct (sheet prints 2027, treated as a typo)</t>
+        </is>
+      </c>
+      <c r="G27" s="20" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="15" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B28" s="16" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="C28" s="16" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="D28" s="18" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E28" s="18" t="n">
+        <v>46319</v>
+      </c>
+      <c r="F28" s="16" t="inlineStr">
+        <is>
+          <t>Close on 4–24 Oct 2026 to renovate electric channel</t>
+        </is>
+      </c>
+      <c r="G28" s="16" t="inlineStr">
+        <is>
+          <t>End back to 24 Oct</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>20E / G.25</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="inlineStr">
+        <is>
+          <t>Gate stopped</t>
+        </is>
+      </c>
+      <c r="D29" s="10" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E29" s="10" t="n">
+        <v>46313</v>
+      </c>
+      <c r="F29" s="9" t="inlineStr">
+        <is>
+          <t>G.25 stops working 5–18 Oct 2026 to change trolley rail</t>
+        </is>
+      </c>
+      <c r="G29" s="9" t="inlineStr">
+        <is>
+          <t>End confirmed as 18 Oct</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="12" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B30" s="13" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="C30" s="13" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="D30" s="22" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E30" s="22" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F30" s="13" t="inlineStr">
+        <is>
+          <t>(no notice – wharf open)</t>
+        </is>
+      </c>
+      <c r="G30" s="13" t="inlineStr">
+        <is>
+          <t>Notice removed: 20C reopened on 5 Oct</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="15" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B31" s="16" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="C31" s="16" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="D31" s="18" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E31" s="18" t="n">
+        <v>46319</v>
+      </c>
+      <c r="F31" s="16" t="inlineStr">
+        <is>
+          <t>Close on 4–24 Oct 2026 to renovate electric channel (but JOSCO LUCKY and MTT BANGKOK are booked at 20D from 06/18)</t>
+        </is>
+      </c>
+      <c r="G31" s="16" t="inlineStr">
+        <is>
+          <t>Unchanged – conflicts with vessel bookings, please confirm</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>20E / G.25</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>Gate stopped</t>
+        </is>
+      </c>
+      <c r="D32" s="10" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E32" s="10" t="n">
+        <v>46313</v>
+      </c>
+      <c r="F32" s="9" t="inlineStr">
+        <is>
+          <t>G.25 stops working 5–18 Oct 2026 to change trolley rail</t>
+        </is>
+      </c>
+      <c r="G32" s="9" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <autoFilter ref="A4:G32"/>
+  <mergeCells count="1">
+    <mergeCell ref="A2:G2"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2110,28 +2975,28 @@
           <t>INFINITY</t>
         </is>
       </c>
-      <c r="C4" s="7" t="n">
+      <c r="C4" s="23" t="n">
         <v>565</v>
       </c>
-      <c r="D4" s="8" t="n">
+      <c r="D4" s="11" t="n">
         <v>46293.29166666666</v>
       </c>
-      <c r="E4" s="8" t="n">
+      <c r="E4" s="11" t="n">
         <v>46293.29166666666</v>
       </c>
-      <c r="F4" s="8" t="n">
+      <c r="F4" s="11" t="n">
         <v>46294.625</v>
       </c>
-      <c r="G4" s="9">
+      <c r="G4" s="26">
         <f>(F4-E4)*24</f>
         <v/>
       </c>
-      <c r="H4" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I4" s="7" t="inlineStr"/>
+      <c r="H4" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I4" s="23" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -2144,28 +3009,28 @@
           <t>SKY CHALLENGE</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C5" s="23" t="n">
         <v>565</v>
       </c>
-      <c r="D5" s="8" t="n">
+      <c r="D5" s="11" t="n">
         <v>46294.45833333334</v>
       </c>
-      <c r="E5" s="8" t="n">
+      <c r="E5" s="11" t="n">
         <v>46294.66666666666</v>
       </c>
-      <c r="F5" s="8" t="n">
+      <c r="F5" s="11" t="n">
         <v>46296.16666666666</v>
       </c>
-      <c r="G5" s="9">
+      <c r="G5" s="26">
         <f>(F5-E5)*24</f>
         <v/>
       </c>
-      <c r="H5" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I5" s="7" t="inlineStr"/>
+      <c r="H5" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I5" s="23" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -2178,28 +3043,28 @@
           <t>CAPE FAWLEY</t>
         </is>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="23" t="n">
         <v>558</v>
       </c>
-      <c r="D6" s="8" t="n">
+      <c r="D6" s="11" t="n">
         <v>46295.875</v>
       </c>
-      <c r="E6" s="8" t="n">
+      <c r="E6" s="11" t="n">
         <v>46296.25</v>
       </c>
-      <c r="F6" s="8" t="n">
+      <c r="F6" s="11" t="n">
         <v>46297.25</v>
       </c>
-      <c r="G6" s="9">
+      <c r="G6" s="26">
         <f>(F6-E6)*24</f>
         <v/>
       </c>
-      <c r="H6" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I6" s="7" t="inlineStr"/>
+      <c r="H6" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I6" s="23" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -2212,28 +3077,28 @@
           <t>KMTC GWANGYANG</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C7" s="23" t="n">
         <v>564</v>
       </c>
-      <c r="D7" s="8" t="n">
+      <c r="D7" s="11" t="n">
         <v>46292.79166666666</v>
       </c>
-      <c r="E7" s="8" t="n">
+      <c r="E7" s="11" t="n">
         <v>46292.79166666666</v>
       </c>
-      <c r="F7" s="8" t="n">
+      <c r="F7" s="11" t="n">
         <v>46294.20833333334</v>
       </c>
-      <c r="G7" s="9">
+      <c r="G7" s="26">
         <f>(F7-E7)*24</f>
         <v/>
       </c>
-      <c r="H7" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I7" s="7" t="inlineStr"/>
+      <c r="H7" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I7" s="23" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -2246,28 +3111,28 @@
           <t>MILLENNIUM BRIGHT</t>
         </is>
       </c>
-      <c r="C8" s="7" t="n">
+      <c r="C8" s="23" t="n">
         <v>564</v>
       </c>
-      <c r="D8" s="8" t="n">
+      <c r="D8" s="11" t="n">
         <v>46293.45833333334</v>
       </c>
-      <c r="E8" s="8" t="n">
+      <c r="E8" s="11" t="n">
         <v>46294.20833333334</v>
       </c>
-      <c r="F8" s="8" t="n">
+      <c r="F8" s="11" t="n">
         <v>46295.16666666666</v>
       </c>
-      <c r="G8" s="9">
+      <c r="G8" s="26">
         <f>(F8-E8)*24</f>
         <v/>
       </c>
-      <c r="H8" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I8" s="7" t="inlineStr"/>
+      <c r="H8" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I8" s="23" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -2280,28 +3145,28 @@
           <t>M ODYSSEY</t>
         </is>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="C9" s="23" t="n">
         <v>449</v>
       </c>
-      <c r="D9" s="8" t="n">
+      <c r="D9" s="11" t="n">
         <v>46295.16666666666</v>
       </c>
-      <c r="E9" s="8" t="n">
+      <c r="E9" s="11" t="n">
         <v>46295.20833333334</v>
       </c>
-      <c r="F9" s="8" t="n">
+      <c r="F9" s="11" t="n">
         <v>46296.70833333334</v>
       </c>
-      <c r="G9" s="9">
+      <c r="G9" s="26">
         <f>(F9-E9)*24</f>
         <v/>
       </c>
-      <c r="H9" s="7" t="inlineStr">
+      <c r="H9" s="23" t="inlineStr">
         <is>
           <t>4A</t>
         </is>
       </c>
-      <c r="I9" s="7" t="inlineStr"/>
+      <c r="I9" s="23" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -2314,28 +3179,28 @@
           <t>BANGKOK</t>
         </is>
       </c>
-      <c r="C10" s="7" t="n">
+      <c r="C10" s="23" t="n">
         <v>551</v>
       </c>
-      <c r="D10" s="8" t="n">
+      <c r="D10" s="11" t="n">
         <v>46292.625</v>
       </c>
-      <c r="E10" s="8" t="n">
+      <c r="E10" s="11" t="n">
         <v>46292.625</v>
       </c>
-      <c r="F10" s="8" t="n">
+      <c r="F10" s="11" t="n">
         <v>46294.58333333334</v>
       </c>
-      <c r="G10" s="9">
+      <c r="G10" s="26">
         <f>(F10-E10)*24</f>
         <v/>
       </c>
-      <c r="H10" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I10" s="7" t="inlineStr"/>
+      <c r="H10" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I10" s="23" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -2348,28 +3213,28 @@
           <t>TS CHIBA</t>
         </is>
       </c>
-      <c r="C11" s="7" t="n">
+      <c r="C11" s="23" t="n">
         <v>485</v>
       </c>
-      <c r="D11" s="8" t="n">
+      <c r="D11" s="11" t="n">
         <v>46293.29166666666</v>
       </c>
-      <c r="E11" s="8" t="n">
+      <c r="E11" s="11" t="n">
         <v>46293.29166666666</v>
       </c>
-      <c r="F11" s="8" t="n">
+      <c r="F11" s="11" t="n">
         <v>46294.16666666666</v>
       </c>
-      <c r="G11" s="9">
+      <c r="G11" s="26">
         <f>(F11-E11)*24</f>
         <v/>
       </c>
-      <c r="H11" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I11" s="7" t="inlineStr"/>
+      <c r="H11" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I11" s="23" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -2382,28 +3247,28 @@
           <t>HOPE C</t>
         </is>
       </c>
-      <c r="C12" s="7" t="n">
+      <c r="C12" s="23" t="n">
         <v>481</v>
       </c>
-      <c r="D12" s="8" t="n">
+      <c r="D12" s="11" t="n">
         <v>46294.70833333334</v>
       </c>
-      <c r="E12" s="8" t="n">
+      <c r="E12" s="11" t="n">
         <v>46294.70833333334</v>
       </c>
-      <c r="F12" s="8" t="n">
+      <c r="F12" s="11" t="n">
         <v>46296.20833333334</v>
       </c>
-      <c r="G12" s="9">
+      <c r="G12" s="26">
         <f>(F12-E12)*24</f>
         <v/>
       </c>
-      <c r="H12" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I12" s="7" t="inlineStr"/>
+      <c r="H12" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I12" s="23" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
@@ -2416,28 +3281,28 @@
           <t>JARU BHUM</t>
         </is>
       </c>
-      <c r="C13" s="10" t="n">
+      <c r="C13" s="17" t="n">
         <v>564</v>
       </c>
-      <c r="D13" s="11" t="n">
+      <c r="D13" s="25" t="n">
         <v>46293.33333333334</v>
       </c>
-      <c r="E13" s="11" t="n">
+      <c r="E13" s="25" t="n">
         <v>46293.33333333334</v>
       </c>
-      <c r="F13" s="11" t="n">
+      <c r="F13" s="25" t="n">
         <v>46294.16666666666</v>
       </c>
-      <c r="G13" s="12">
+      <c r="G13" s="27">
         <f>(F13-E13)*24</f>
         <v/>
       </c>
-      <c r="H13" s="10" t="inlineStr">
+      <c r="H13" s="17" t="inlineStr">
         <is>
           <t>7B</t>
         </is>
       </c>
-      <c r="I13" s="10" t="inlineStr">
+      <c r="I13" s="17" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -2454,28 +3319,28 @@
           <t>MITRA BHUM</t>
         </is>
       </c>
-      <c r="C14" s="7" t="n">
+      <c r="C14" s="23" t="n">
         <v>485</v>
       </c>
-      <c r="D14" s="8" t="n">
+      <c r="D14" s="11" t="n">
         <v>46294.95833333334</v>
       </c>
-      <c r="E14" s="8" t="n">
+      <c r="E14" s="11" t="n">
         <v>46295.20833333334</v>
       </c>
-      <c r="F14" s="8" t="n">
+      <c r="F14" s="11" t="n">
         <v>46295.75</v>
       </c>
-      <c r="G14" s="9">
+      <c r="G14" s="26">
         <f>(F14-E14)*24</f>
         <v/>
       </c>
-      <c r="H14" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I14" s="7" t="inlineStr"/>
+      <c r="H14" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I14" s="23" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2567,28 +3432,28 @@
           <t>INFINITY</t>
         </is>
       </c>
-      <c r="C4" s="7" t="n">
+      <c r="C4" s="23" t="n">
         <v>565</v>
       </c>
-      <c r="D4" s="8" t="n">
+      <c r="D4" s="11" t="n">
         <v>46292.75</v>
       </c>
-      <c r="E4" s="8" t="n">
+      <c r="E4" s="11" t="n">
         <v>46293.20833333334</v>
       </c>
-      <c r="F4" s="8" t="n">
+      <c r="F4" s="11" t="n">
         <v>46294.625</v>
       </c>
-      <c r="G4" s="9">
+      <c r="G4" s="26">
         <f>(F4-E4)*24</f>
         <v/>
       </c>
-      <c r="H4" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I4" s="7" t="inlineStr"/>
+      <c r="H4" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I4" s="23" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -2601,28 +3466,28 @@
           <t>SKY CHALLENGE</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C5" s="23" t="n">
         <v>565</v>
       </c>
-      <c r="D5" s="8" t="n">
+      <c r="D5" s="11" t="n">
         <v>46294.33333333334</v>
       </c>
-      <c r="E5" s="8" t="n">
+      <c r="E5" s="11" t="n">
         <v>46294.66666666666</v>
       </c>
-      <c r="F5" s="8" t="n">
+      <c r="F5" s="11" t="n">
         <v>46296.16666666666</v>
       </c>
-      <c r="G5" s="9">
+      <c r="G5" s="26">
         <f>(F5-E5)*24</f>
         <v/>
       </c>
-      <c r="H5" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I5" s="7" t="inlineStr"/>
+      <c r="H5" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I5" s="23" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -2635,28 +3500,28 @@
           <t>KHARIS HERITAGE</t>
         </is>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="23" t="n">
         <v>482</v>
       </c>
-      <c r="D6" s="8" t="n">
+      <c r="D6" s="11" t="n">
         <v>46296.29166666666</v>
       </c>
-      <c r="E6" s="8" t="n">
+      <c r="E6" s="11" t="n">
         <v>46296.29166666666</v>
       </c>
-      <c r="F6" s="8" t="n">
+      <c r="F6" s="11" t="n">
         <v>46297.25</v>
       </c>
-      <c r="G6" s="9">
+      <c r="G6" s="26">
         <f>(F6-E6)*24</f>
         <v/>
       </c>
-      <c r="H6" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I6" s="7" t="inlineStr"/>
+      <c r="H6" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I6" s="23" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -2669,28 +3534,28 @@
           <t>MILLENNIUM BRIGHT</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C7" s="23" t="n">
         <v>564</v>
       </c>
-      <c r="D7" s="8" t="n">
+      <c r="D7" s="11" t="n">
         <v>46293.45833333334</v>
       </c>
-      <c r="E7" s="8" t="n">
+      <c r="E7" s="11" t="n">
         <v>46294.20833333334</v>
       </c>
-      <c r="F7" s="8" t="n">
+      <c r="F7" s="11" t="n">
         <v>46295.16666666666</v>
       </c>
-      <c r="G7" s="9">
+      <c r="G7" s="26">
         <f>(F7-E7)*24</f>
         <v/>
       </c>
-      <c r="H7" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I7" s="7" t="inlineStr"/>
+      <c r="H7" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I7" s="23" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -2703,28 +3568,28 @@
           <t>M ODYSSEY</t>
         </is>
       </c>
-      <c r="C8" s="7" t="n">
+      <c r="C8" s="23" t="n">
         <v>449</v>
       </c>
-      <c r="D8" s="8" t="n">
+      <c r="D8" s="11" t="n">
         <v>46295.16666666666</v>
       </c>
-      <c r="E8" s="8" t="n">
+      <c r="E8" s="11" t="n">
         <v>46295.20833333334</v>
       </c>
-      <c r="F8" s="8" t="n">
+      <c r="F8" s="11" t="n">
         <v>46296.20833333334</v>
       </c>
-      <c r="G8" s="9">
+      <c r="G8" s="26">
         <f>(F8-E8)*24</f>
         <v/>
       </c>
-      <c r="H8" s="7" t="inlineStr">
+      <c r="H8" s="23" t="inlineStr">
         <is>
           <t>4A</t>
         </is>
       </c>
-      <c r="I8" s="7" t="inlineStr"/>
+      <c r="I8" s="23" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -2737,28 +3602,28 @@
           <t>CAPE FAWLEY</t>
         </is>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="C9" s="23" t="n">
         <v>558</v>
       </c>
-      <c r="D9" s="8" t="n">
+      <c r="D9" s="11" t="n">
         <v>46295.875</v>
       </c>
-      <c r="E9" s="8" t="n">
+      <c r="E9" s="11" t="n">
         <v>46296.25</v>
       </c>
-      <c r="F9" s="8" t="n">
+      <c r="F9" s="11" t="n">
         <v>46297.25</v>
       </c>
-      <c r="G9" s="9">
+      <c r="G9" s="26">
         <f>(F9-E9)*24</f>
         <v/>
       </c>
-      <c r="H9" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I9" s="7" t="inlineStr"/>
+      <c r="H9" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I9" s="23" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -2771,28 +3636,28 @@
           <t>BANGKOK</t>
         </is>
       </c>
-      <c r="C10" s="7" t="n">
+      <c r="C10" s="23" t="n">
         <v>551</v>
       </c>
-      <c r="D10" s="8" t="n">
+      <c r="D10" s="11" t="n">
         <v>46292.54166666666</v>
       </c>
-      <c r="E10" s="8" t="n">
+      <c r="E10" s="11" t="n">
         <v>46292.625</v>
       </c>
-      <c r="F10" s="8" t="n">
+      <c r="F10" s="11" t="n">
         <v>46294.58333333334</v>
       </c>
-      <c r="G10" s="9">
+      <c r="G10" s="26">
         <f>(F10-E10)*24</f>
         <v/>
       </c>
-      <c r="H10" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I10" s="7" t="inlineStr"/>
+      <c r="H10" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I10" s="23" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -2805,28 +3670,28 @@
           <t>MITRA BHUM</t>
         </is>
       </c>
-      <c r="C11" s="7" t="n">
+      <c r="C11" s="23" t="n">
         <v>485</v>
       </c>
-      <c r="D11" s="8" t="n">
+      <c r="D11" s="11" t="n">
         <v>46295.125</v>
       </c>
-      <c r="E11" s="8" t="n">
+      <c r="E11" s="11" t="n">
         <v>46295.20833333334</v>
       </c>
-      <c r="F11" s="8" t="n">
+      <c r="F11" s="11" t="n">
         <v>46295.75</v>
       </c>
-      <c r="G11" s="9">
+      <c r="G11" s="26">
         <f>(F11-E11)*24</f>
         <v/>
       </c>
-      <c r="H11" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I11" s="7" t="inlineStr"/>
+      <c r="H11" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I11" s="23" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -2839,28 +3704,28 @@
           <t>HOPE C</t>
         </is>
       </c>
-      <c r="C12" s="7" t="n">
+      <c r="C12" s="23" t="n">
         <v>481</v>
       </c>
-      <c r="D12" s="8" t="n">
+      <c r="D12" s="11" t="n">
         <v>46294.70833333334</v>
       </c>
-      <c r="E12" s="8" t="n">
+      <c r="E12" s="11" t="n">
         <v>46294.70833333334</v>
       </c>
-      <c r="F12" s="8" t="n">
+      <c r="F12" s="11" t="n">
         <v>46295.66666666666</v>
       </c>
-      <c r="G12" s="9">
+      <c r="G12" s="26">
         <f>(F12-E12)*24</f>
         <v/>
       </c>
-      <c r="H12" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I12" s="7" t="inlineStr"/>
+      <c r="H12" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I12" s="23" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -2873,28 +3738,28 @@
           <t>ALS SUMIRE</t>
         </is>
       </c>
-      <c r="C13" s="7" t="n">
+      <c r="C13" s="23" t="n">
         <v>537</v>
       </c>
-      <c r="D13" s="8" t="n">
+      <c r="D13" s="11" t="n">
         <v>46296.54166666666</v>
       </c>
-      <c r="E13" s="8" t="n">
+      <c r="E13" s="11" t="n">
         <v>46296.70833333334</v>
       </c>
-      <c r="F13" s="8" t="n">
+      <c r="F13" s="11" t="n">
         <v>46297.70833333334</v>
       </c>
-      <c r="G13" s="9">
+      <c r="G13" s="26">
         <f>(F13-E13)*24</f>
         <v/>
       </c>
-      <c r="H13" s="7" t="inlineStr">
+      <c r="H13" s="23" t="inlineStr">
         <is>
           <t>1C</t>
         </is>
       </c>
-      <c r="I13" s="7" t="inlineStr"/>
+      <c r="I13" s="23" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2986,28 +3851,28 @@
           <t>SKY CHALLENGE</t>
         </is>
       </c>
-      <c r="C4" s="7" t="n">
+      <c r="C4" s="23" t="n">
         <v>565</v>
       </c>
-      <c r="D4" s="8" t="n">
+      <c r="D4" s="11" t="n">
         <v>46294.33333333334</v>
       </c>
-      <c r="E4" s="8" t="n">
+      <c r="E4" s="11" t="n">
         <v>46294.66666666666</v>
       </c>
-      <c r="F4" s="8" t="n">
+      <c r="F4" s="11" t="n">
         <v>46296.16666666666</v>
       </c>
-      <c r="G4" s="9">
+      <c r="G4" s="26">
         <f>(F4-E4)*24</f>
         <v/>
       </c>
-      <c r="H4" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I4" s="7" t="inlineStr"/>
+      <c r="H4" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I4" s="23" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -3020,28 +3885,28 @@
           <t>CAPE FAWLEY</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C5" s="23" t="n">
         <v>558</v>
       </c>
-      <c r="D5" s="8" t="n">
+      <c r="D5" s="11" t="n">
         <v>46295.875</v>
       </c>
-      <c r="E5" s="8" t="n">
+      <c r="E5" s="11" t="n">
         <v>46296.25</v>
       </c>
-      <c r="F5" s="8" t="n">
+      <c r="F5" s="11" t="n">
         <v>46297.25</v>
       </c>
-      <c r="G5" s="9">
+      <c r="G5" s="26">
         <f>(F5-E5)*24</f>
         <v/>
       </c>
-      <c r="H5" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I5" s="7" t="inlineStr"/>
+      <c r="H5" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I5" s="23" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -3054,28 +3919,28 @@
           <t>KMTC BANGKOK</t>
         </is>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="23" t="n">
         <v>565</v>
       </c>
-      <c r="D6" s="8" t="n">
+      <c r="D6" s="11" t="n">
         <v>46297.25</v>
       </c>
-      <c r="E6" s="8" t="n">
+      <c r="E6" s="11" t="n">
         <v>46297.33333333334</v>
       </c>
-      <c r="F6" s="8" t="n">
+      <c r="F6" s="11" t="n">
         <v>46298.70833333334</v>
       </c>
-      <c r="G6" s="9">
+      <c r="G6" s="26">
         <f>(F6-E6)*24</f>
         <v/>
       </c>
-      <c r="H6" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I6" s="7" t="inlineStr"/>
+      <c r="H6" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I6" s="23" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -3088,28 +3953,28 @@
           <t>M ODYSSEY</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C7" s="23" t="n">
         <v>449</v>
       </c>
-      <c r="D7" s="8" t="n">
+      <c r="D7" s="11" t="n">
         <v>46295.16666666666</v>
       </c>
-      <c r="E7" s="8" t="n">
+      <c r="E7" s="11" t="n">
         <v>46295.20833333334</v>
       </c>
-      <c r="F7" s="8" t="n">
+      <c r="F7" s="11" t="n">
         <v>46296.20833333334</v>
       </c>
-      <c r="G7" s="9">
+      <c r="G7" s="26">
         <f>(F7-E7)*24</f>
         <v/>
       </c>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="H7" s="23" t="inlineStr">
         <is>
           <t>4A</t>
         </is>
       </c>
-      <c r="I7" s="7" t="inlineStr"/>
+      <c r="I7" s="23" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -3122,28 +3987,28 @@
           <t>KHARIS HERITAGE</t>
         </is>
       </c>
-      <c r="C8" s="10" t="n">
+      <c r="C8" s="17" t="n">
         <v>482</v>
       </c>
-      <c r="D8" s="11" t="n">
+      <c r="D8" s="25" t="n">
         <v>46296.45833333334</v>
       </c>
-      <c r="E8" s="11" t="n">
+      <c r="E8" s="25" t="n">
         <v>46296.70833333334</v>
       </c>
-      <c r="F8" s="11" t="n">
+      <c r="F8" s="25" t="n">
         <v>46297.70833333334</v>
       </c>
-      <c r="G8" s="12">
+      <c r="G8" s="27">
         <f>(F8-E8)*24</f>
         <v/>
       </c>
-      <c r="H8" s="10" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I8" s="10" t="inlineStr">
+      <c r="H8" s="17" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I8" s="17" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3160,28 +4025,28 @@
           <t>ALS SUMIRE</t>
         </is>
       </c>
-      <c r="C9" s="10" t="n">
+      <c r="C9" s="17" t="n">
         <v>537</v>
       </c>
-      <c r="D9" s="11" t="n">
+      <c r="D9" s="25" t="n">
         <v>46296.70833333334</v>
       </c>
-      <c r="E9" s="11" t="n">
+      <c r="E9" s="25" t="n">
         <v>46296.70833333334</v>
       </c>
-      <c r="F9" s="11" t="n">
+      <c r="F9" s="25" t="n">
         <v>46297.70833333334</v>
       </c>
-      <c r="G9" s="12">
+      <c r="G9" s="27">
         <f>(F9-E9)*24</f>
         <v/>
       </c>
-      <c r="H9" s="10" t="inlineStr">
+      <c r="H9" s="17" t="inlineStr">
         <is>
           <t>1C</t>
         </is>
       </c>
-      <c r="I9" s="10" t="inlineStr">
+      <c r="I9" s="17" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3198,28 +4063,28 @@
           <t>MITRA BHUM</t>
         </is>
       </c>
-      <c r="C10" s="7" t="n">
+      <c r="C10" s="23" t="n">
         <v>485</v>
       </c>
-      <c r="D10" s="8" t="n">
+      <c r="D10" s="11" t="n">
         <v>46295.125</v>
       </c>
-      <c r="E10" s="8" t="n">
+      <c r="E10" s="11" t="n">
         <v>46295.20833333334</v>
       </c>
-      <c r="F10" s="8" t="n">
+      <c r="F10" s="11" t="n">
         <v>46295.75</v>
       </c>
-      <c r="G10" s="9">
+      <c r="G10" s="26">
         <f>(F10-E10)*24</f>
         <v/>
       </c>
-      <c r="H10" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I10" s="7" t="inlineStr"/>
+      <c r="H10" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I10" s="23" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -3232,28 +4097,28 @@
           <t>HOPE C</t>
         </is>
       </c>
-      <c r="C11" s="7" t="n">
+      <c r="C11" s="23" t="n">
         <v>481</v>
       </c>
-      <c r="D11" s="8" t="n">
+      <c r="D11" s="11" t="n">
         <v>46294.70833333334</v>
       </c>
-      <c r="E11" s="8" t="n">
+      <c r="E11" s="11" t="n">
         <v>46294.70833333334</v>
       </c>
-      <c r="F11" s="8" t="n">
+      <c r="F11" s="11" t="n">
         <v>46295.66666666666</v>
       </c>
-      <c r="G11" s="9">
+      <c r="G11" s="26">
         <f>(F11-E11)*24</f>
         <v/>
       </c>
-      <c r="H11" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I11" s="7" t="inlineStr"/>
+      <c r="H11" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I11" s="23" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -3266,28 +4131,28 @@
           <t>WAN HAI 278</t>
         </is>
       </c>
-      <c r="C12" s="7" t="n">
+      <c r="C12" s="23" t="n">
         <v>564</v>
       </c>
-      <c r="D12" s="8" t="n">
+      <c r="D12" s="11" t="n">
         <v>46297.375</v>
       </c>
-      <c r="E12" s="8" t="n">
+      <c r="E12" s="11" t="n">
         <v>46297.375</v>
       </c>
-      <c r="F12" s="8" t="n">
+      <c r="F12" s="11" t="n">
         <v>46299.41666666666</v>
       </c>
-      <c r="G12" s="9">
+      <c r="G12" s="26">
         <f>(F12-E12)*24</f>
         <v/>
       </c>
-      <c r="H12" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I12" s="7" t="inlineStr"/>
+      <c r="H12" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I12" s="23" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3379,28 +4244,28 @@
           <t>CAPE FAWLEY</t>
         </is>
       </c>
-      <c r="C4" s="7" t="n">
+      <c r="C4" s="23" t="n">
         <v>558</v>
       </c>
-      <c r="D4" s="8" t="n">
+      <c r="D4" s="11" t="n">
         <v>46295.875</v>
       </c>
-      <c r="E4" s="8" t="n">
+      <c r="E4" s="11" t="n">
         <v>46296.25</v>
       </c>
-      <c r="F4" s="8" t="n">
+      <c r="F4" s="11" t="n">
         <v>46297.25</v>
       </c>
-      <c r="G4" s="9">
+      <c r="G4" s="26">
         <f>(F4-E4)*24</f>
         <v/>
       </c>
-      <c r="H4" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I4" s="7" t="inlineStr"/>
+      <c r="H4" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I4" s="23" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -3413,28 +4278,28 @@
           <t>KMTC BANGKOK</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C5" s="23" t="n">
         <v>565</v>
       </c>
-      <c r="D5" s="8" t="n">
+      <c r="D5" s="11" t="n">
         <v>46297.25</v>
       </c>
-      <c r="E5" s="8" t="n">
+      <c r="E5" s="11" t="n">
         <v>46297.33333333334</v>
       </c>
-      <c r="F5" s="8" t="n">
+      <c r="F5" s="11" t="n">
         <v>46298.70833333334</v>
       </c>
-      <c r="G5" s="9">
+      <c r="G5" s="26">
         <f>(F5-E5)*24</f>
         <v/>
       </c>
-      <c r="H5" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I5" s="7" t="inlineStr"/>
+      <c r="H5" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I5" s="23" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -3447,28 +4312,28 @@
           <t>KHARIS HERITAGE</t>
         </is>
       </c>
-      <c r="C6" s="10" t="n">
+      <c r="C6" s="17" t="n">
         <v>482</v>
       </c>
-      <c r="D6" s="11" t="n">
+      <c r="D6" s="25" t="n">
         <v>46296.5</v>
       </c>
-      <c r="E6" s="11" t="n">
+      <c r="E6" s="25" t="n">
         <v>46296.70833333334</v>
       </c>
-      <c r="F6" s="11" t="n">
+      <c r="F6" s="25" t="n">
         <v>46297.70833333334</v>
       </c>
-      <c r="G6" s="12">
+      <c r="G6" s="27">
         <f>(F6-E6)*24</f>
         <v/>
       </c>
-      <c r="H6" s="10" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I6" s="10" t="inlineStr">
+      <c r="H6" s="17" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I6" s="17" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3485,28 +4350,28 @@
           <t>ZHONG GU BEI HAI</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C7" s="23" t="n">
         <v>561</v>
       </c>
-      <c r="D7" s="8" t="n">
+      <c r="D7" s="11" t="n">
         <v>46298.91666666666</v>
       </c>
-      <c r="E7" s="8" t="n">
+      <c r="E7" s="11" t="n">
         <v>46299.375</v>
       </c>
-      <c r="F7" s="8" t="n">
+      <c r="F7" s="11" t="n">
         <v>46300.66666666666</v>
       </c>
-      <c r="G7" s="9">
+      <c r="G7" s="26">
         <f>(F7-E7)*24</f>
         <v/>
       </c>
-      <c r="H7" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I7" s="7" t="inlineStr"/>
+      <c r="H7" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I7" s="23" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -3519,28 +4384,28 @@
           <t>YM IMPROVEMENT</t>
         </is>
       </c>
-      <c r="C8" s="7" t="n">
+      <c r="C8" s="23" t="n">
         <v>564</v>
       </c>
-      <c r="D8" s="8" t="n">
+      <c r="D8" s="11" t="n">
         <v>46298.83333333334</v>
       </c>
-      <c r="E8" s="8" t="n">
+      <c r="E8" s="11" t="n">
         <v>46298.83333333334</v>
       </c>
-      <c r="F8" s="8" t="n">
+      <c r="F8" s="11" t="n">
         <v>46300.41666666666</v>
       </c>
-      <c r="G8" s="9">
+      <c r="G8" s="26">
         <f>(F8-E8)*24</f>
         <v/>
       </c>
-      <c r="H8" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I8" s="7" t="inlineStr"/>
+      <c r="H8" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I8" s="23" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -3553,28 +4418,28 @@
           <t>ALS SUMIRE</t>
         </is>
       </c>
-      <c r="C9" s="10" t="n">
+      <c r="C9" s="17" t="n">
         <v>537</v>
       </c>
-      <c r="D9" s="11" t="n">
+      <c r="D9" s="25" t="n">
         <v>46296.70833333334</v>
       </c>
-      <c r="E9" s="11" t="n">
+      <c r="E9" s="25" t="n">
         <v>46296.70833333334</v>
       </c>
-      <c r="F9" s="11" t="n">
+      <c r="F9" s="25" t="n">
         <v>46297.70833333334</v>
       </c>
-      <c r="G9" s="12">
+      <c r="G9" s="27">
         <f>(F9-E9)*24</f>
         <v/>
       </c>
-      <c r="H9" s="10" t="inlineStr">
+      <c r="H9" s="17" t="inlineStr">
         <is>
           <t>1C</t>
         </is>
       </c>
-      <c r="I9" s="10" t="inlineStr">
+      <c r="I9" s="17" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3591,28 +4456,28 @@
           <t>RESURGENCE</t>
         </is>
       </c>
-      <c r="C10" s="7" t="n">
+      <c r="C10" s="23" t="n">
         <v>458</v>
       </c>
-      <c r="D10" s="8" t="n">
+      <c r="D10" s="11" t="n">
         <v>46298.75</v>
       </c>
-      <c r="E10" s="8" t="n">
+      <c r="E10" s="11" t="n">
         <v>46298.75</v>
       </c>
-      <c r="F10" s="8" t="n">
+      <c r="F10" s="11" t="n">
         <v>46299.83333333334</v>
       </c>
-      <c r="G10" s="9">
+      <c r="G10" s="26">
         <f>(F10-E10)*24</f>
         <v/>
       </c>
-      <c r="H10" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I10" s="7" t="inlineStr"/>
+      <c r="H10" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I10" s="23" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -3625,28 +4490,28 @@
           <t>WAN HAI 278</t>
         </is>
       </c>
-      <c r="C11" s="7" t="n">
+      <c r="C11" s="23" t="n">
         <v>564</v>
       </c>
-      <c r="D11" s="8" t="n">
+      <c r="D11" s="11" t="n">
         <v>46297.375</v>
       </c>
-      <c r="E11" s="8" t="n">
+      <c r="E11" s="11" t="n">
         <v>46297.375</v>
       </c>
-      <c r="F11" s="8" t="n">
+      <c r="F11" s="11" t="n">
         <v>46299.41666666666</v>
       </c>
-      <c r="G11" s="9">
+      <c r="G11" s="26">
         <f>(F11-E11)*24</f>
         <v/>
       </c>
-      <c r="H11" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I11" s="7" t="inlineStr"/>
+      <c r="H11" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I11" s="23" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3738,28 +4603,28 @@
           <t>CAPE FAWLEY</t>
         </is>
       </c>
-      <c r="C4" s="7" t="n">
+      <c r="C4" s="23" t="n">
         <v>558</v>
       </c>
-      <c r="D4" s="8" t="n">
+      <c r="D4" s="11" t="n">
         <v>46295.875</v>
       </c>
-      <c r="E4" s="8" t="n">
+      <c r="E4" s="11" t="n">
         <v>46296.25</v>
       </c>
-      <c r="F4" s="8" t="n">
+      <c r="F4" s="11" t="n">
         <v>46297.625</v>
       </c>
-      <c r="G4" s="9">
+      <c r="G4" s="26">
         <f>(F4-E4)*24</f>
         <v/>
       </c>
-      <c r="H4" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I4" s="7" t="inlineStr"/>
+      <c r="H4" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I4" s="23" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -3772,28 +4637,28 @@
           <t>RESURGENCE</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C5" s="23" t="n">
         <v>458</v>
       </c>
-      <c r="D5" s="8" t="n">
+      <c r="D5" s="11" t="n">
         <v>46298.54166666666</v>
       </c>
-      <c r="E5" s="8" t="n">
+      <c r="E5" s="11" t="n">
         <v>46298.54166666666</v>
       </c>
-      <c r="F5" s="8" t="n">
+      <c r="F5" s="11" t="n">
         <v>46299.5</v>
       </c>
-      <c r="G5" s="9">
+      <c r="G5" s="26">
         <f>(F5-E5)*24</f>
         <v/>
       </c>
-      <c r="H5" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I5" s="7" t="inlineStr"/>
+      <c r="H5" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I5" s="23" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -3806,28 +4671,28 @@
           <t>ZHONG GU BEI HAI</t>
         </is>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="23" t="n">
         <v>561</v>
       </c>
-      <c r="D6" s="8" t="n">
+      <c r="D6" s="11" t="n">
         <v>46299.375</v>
       </c>
-      <c r="E6" s="8" t="n">
+      <c r="E6" s="11" t="n">
         <v>46299.45833333334</v>
       </c>
-      <c r="F6" s="8" t="n">
+      <c r="F6" s="11" t="n">
         <v>46301.45833333334</v>
       </c>
-      <c r="G6" s="9">
+      <c r="G6" s="26">
         <f>(F6-E6)*24</f>
         <v/>
       </c>
-      <c r="H6" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I6" s="7" t="inlineStr"/>
+      <c r="H6" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I6" s="23" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -3840,28 +4705,28 @@
           <t>KHARIS HERITAGE</t>
         </is>
       </c>
-      <c r="C7" s="10" t="n">
+      <c r="C7" s="17" t="n">
         <v>482</v>
       </c>
-      <c r="D7" s="11" t="n">
+      <c r="D7" s="25" t="n">
         <v>46296.45833333334</v>
       </c>
-      <c r="E7" s="11" t="n">
+      <c r="E7" s="25" t="n">
         <v>46296.75</v>
       </c>
-      <c r="F7" s="11" t="n">
+      <c r="F7" s="25" t="n">
         <v>46297.70833333334</v>
       </c>
-      <c r="G7" s="12">
+      <c r="G7" s="27">
         <f>(F7-E7)*24</f>
         <v/>
       </c>
-      <c r="H7" s="10" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I7" s="10" t="inlineStr">
+      <c r="H7" s="17" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I7" s="17" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3878,28 +4743,28 @@
           <t>YM IMPROVEMENT</t>
         </is>
       </c>
-      <c r="C8" s="7" t="n">
+      <c r="C8" s="23" t="n">
         <v>564</v>
       </c>
-      <c r="D8" s="8" t="n">
+      <c r="D8" s="11" t="n">
         <v>46298.83333333334</v>
       </c>
-      <c r="E8" s="8" t="n">
+      <c r="E8" s="11" t="n">
         <v>46298.83333333334</v>
       </c>
-      <c r="F8" s="8" t="n">
+      <c r="F8" s="11" t="n">
         <v>46300.41666666666</v>
       </c>
-      <c r="G8" s="9">
+      <c r="G8" s="26">
         <f>(F8-E8)*24</f>
         <v/>
       </c>
-      <c r="H8" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I8" s="7" t="inlineStr"/>
+      <c r="H8" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I8" s="23" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -3912,28 +4777,28 @@
           <t>JOSCO LUCKY</t>
         </is>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="C9" s="23" t="n">
         <v>564</v>
       </c>
-      <c r="D9" s="8" t="n">
+      <c r="D9" s="11" t="n">
         <v>46300.91666666666</v>
       </c>
-      <c r="E9" s="8" t="n">
+      <c r="E9" s="11" t="n">
         <v>46301.5</v>
       </c>
-      <c r="F9" s="8" t="n">
+      <c r="F9" s="11" t="n">
         <v>46302.54166666666</v>
       </c>
-      <c r="G9" s="9">
+      <c r="G9" s="26">
         <f>(F9-E9)*24</f>
         <v/>
       </c>
-      <c r="H9" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I9" s="7" t="inlineStr"/>
+      <c r="H9" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I9" s="23" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -3946,28 +4811,28 @@
           <t>SAWASDEE DENEB</t>
         </is>
       </c>
-      <c r="C10" s="7" t="n">
+      <c r="C10" s="23" t="n">
         <v>564</v>
       </c>
-      <c r="D10" s="8" t="n">
+      <c r="D10" s="11" t="n">
         <v>46300</v>
       </c>
-      <c r="E10" s="8" t="n">
+      <c r="E10" s="11" t="n">
         <v>46300.5</v>
       </c>
-      <c r="F10" s="8" t="n">
+      <c r="F10" s="11" t="n">
         <v>46302.5</v>
       </c>
-      <c r="G10" s="9">
+      <c r="G10" s="26">
         <f>(F10-E10)*24</f>
         <v/>
       </c>
-      <c r="H10" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I10" s="7" t="inlineStr"/>
+      <c r="H10" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I10" s="23" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -3980,28 +4845,28 @@
           <t>ALS SUMIRE</t>
         </is>
       </c>
-      <c r="C11" s="10" t="n">
+      <c r="C11" s="17" t="n">
         <v>537</v>
       </c>
-      <c r="D11" s="11" t="n">
+      <c r="D11" s="25" t="n">
         <v>46296.25</v>
       </c>
-      <c r="E11" s="11" t="n">
+      <c r="E11" s="25" t="n">
         <v>46296.66666666666</v>
       </c>
-      <c r="F11" s="11" t="n">
+      <c r="F11" s="25" t="n">
         <v>46297.70833333334</v>
       </c>
-      <c r="G11" s="12">
+      <c r="G11" s="27">
         <f>(F11-E11)*24</f>
         <v/>
       </c>
-      <c r="H11" s="10" t="inlineStr">
+      <c r="H11" s="17" t="inlineStr">
         <is>
           <t>1C</t>
         </is>
       </c>
-      <c r="I11" s="10" t="inlineStr">
+      <c r="I11" s="17" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4018,28 +4883,28 @@
           <t>HARI BHUM (Barge)</t>
         </is>
       </c>
-      <c r="C12" s="7" t="n">
+      <c r="C12" s="23" t="n">
         <v>259</v>
       </c>
-      <c r="D12" s="8" t="n">
+      <c r="D12" s="11" t="n">
         <v>46298.20833333334</v>
       </c>
-      <c r="E12" s="8" t="n">
+      <c r="E12" s="11" t="n">
         <v>46298.20833333334</v>
       </c>
-      <c r="F12" s="8" t="n">
+      <c r="F12" s="11" t="n">
         <v>46298.66666666666</v>
       </c>
-      <c r="G12" s="9">
+      <c r="G12" s="26">
         <f>(F12-E12)*24</f>
         <v/>
       </c>
-      <c r="H12" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I12" s="7" t="inlineStr"/>
+      <c r="H12" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I12" s="23" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -4052,28 +4917,28 @@
           <t>WAN HAI 278</t>
         </is>
       </c>
-      <c r="C13" s="7" t="n">
+      <c r="C13" s="23" t="n">
         <v>564</v>
       </c>
-      <c r="D13" s="8" t="n">
+      <c r="D13" s="11" t="n">
         <v>46297.75</v>
       </c>
-      <c r="E13" s="8" t="n">
+      <c r="E13" s="11" t="n">
         <v>46298.41666666666</v>
       </c>
-      <c r="F13" s="8" t="n">
+      <c r="F13" s="11" t="n">
         <v>46300.45833333334</v>
       </c>
-      <c r="G13" s="9">
+      <c r="G13" s="26">
         <f>(F13-E13)*24</f>
         <v/>
       </c>
-      <c r="H13" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I13" s="7" t="inlineStr"/>
+      <c r="H13" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I13" s="23" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -4086,28 +4951,28 @@
           <t>KMTC BANGKOK</t>
         </is>
       </c>
-      <c r="C14" s="7" t="n">
+      <c r="C14" s="23" t="n">
         <v>565</v>
       </c>
-      <c r="D14" s="8" t="n">
+      <c r="D14" s="11" t="n">
         <v>46297.29166666666</v>
       </c>
-      <c r="E14" s="8" t="n">
+      <c r="E14" s="11" t="n">
         <v>46297.33333333334</v>
       </c>
-      <c r="F14" s="8" t="n">
+      <c r="F14" s="11" t="n">
         <v>46298.70833333334</v>
       </c>
-      <c r="G14" s="9">
+      <c r="G14" s="26">
         <f>(F14-E14)*24</f>
         <v/>
       </c>
-      <c r="H14" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I14" s="7" t="inlineStr"/>
+      <c r="H14" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I14" s="23" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -4120,28 +4985,28 @@
           <t>XIN MING ZHOU 98</t>
         </is>
       </c>
-      <c r="C15" s="7" t="n">
+      <c r="C15" s="23" t="n">
         <v>564</v>
       </c>
-      <c r="D15" s="8" t="n">
+      <c r="D15" s="11" t="n">
         <v>46299.375</v>
       </c>
-      <c r="E15" s="8" t="n">
+      <c r="E15" s="11" t="n">
         <v>46299.375</v>
       </c>
-      <c r="F15" s="8" t="n">
+      <c r="F15" s="11" t="n">
         <v>46300.375</v>
       </c>
-      <c r="G15" s="9">
+      <c r="G15" s="26">
         <f>(F15-E15)*24</f>
         <v/>
       </c>
-      <c r="H15" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I15" s="7" t="inlineStr"/>
+      <c r="H15" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I15" s="23" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4233,28 +5098,28 @@
           <t>RESURGENCE</t>
         </is>
       </c>
-      <c r="C4" s="7" t="n">
+      <c r="C4" s="23" t="n">
         <v>458</v>
       </c>
-      <c r="D4" s="8" t="n">
+      <c r="D4" s="11" t="n">
         <v>46298.5</v>
       </c>
-      <c r="E4" s="8" t="n">
+      <c r="E4" s="11" t="n">
         <v>46298.5</v>
       </c>
-      <c r="F4" s="8" t="n">
+      <c r="F4" s="11" t="n">
         <v>46299.70833333334</v>
       </c>
-      <c r="G4" s="9">
+      <c r="G4" s="26">
         <f>(F4-E4)*24</f>
         <v/>
       </c>
-      <c r="H4" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I4" s="7" t="inlineStr"/>
+      <c r="H4" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I4" s="23" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -4267,28 +5132,28 @@
           <t>ZHONG GU BEI HAI</t>
         </is>
       </c>
-      <c r="C5" s="10" t="n">
+      <c r="C5" s="17" t="n">
         <v>561</v>
       </c>
-      <c r="D5" s="11" t="n">
+      <c r="D5" s="25" t="n">
         <v>46299.375</v>
       </c>
-      <c r="E5" s="11" t="n">
+      <c r="E5" s="25" t="n">
         <v>46299.625</v>
       </c>
-      <c r="F5" s="11" t="n">
+      <c r="F5" s="25" t="n">
         <v>46301.41666666666</v>
       </c>
-      <c r="G5" s="12">
+      <c r="G5" s="27">
         <f>(F5-E5)*24</f>
         <v/>
       </c>
-      <c r="H5" s="10" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I5" s="10" t="inlineStr">
+      <c r="H5" s="17" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I5" s="17" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4305,28 +5170,28 @@
           <t>YM IMPROVEMENT</t>
         </is>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="23" t="n">
         <v>564</v>
       </c>
-      <c r="D6" s="8" t="n">
+      <c r="D6" s="11" t="n">
         <v>46298.95833333334</v>
       </c>
-      <c r="E6" s="8" t="n">
+      <c r="E6" s="11" t="n">
         <v>46299.41666666666</v>
       </c>
-      <c r="F6" s="8" t="n">
+      <c r="F6" s="11" t="n">
         <v>46300.5</v>
       </c>
-      <c r="G6" s="9">
+      <c r="G6" s="26">
         <f>(F6-E6)*24</f>
         <v/>
       </c>
-      <c r="H6" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I6" s="7" t="inlineStr"/>
+      <c r="H6" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I6" s="23" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -4339,28 +5204,28 @@
           <t>JOSCO LUCKY</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C7" s="23" t="n">
         <v>564</v>
       </c>
-      <c r="D7" s="8" t="n">
+      <c r="D7" s="11" t="n">
         <v>46300.91666666666</v>
       </c>
-      <c r="E7" s="8" t="n">
+      <c r="E7" s="11" t="n">
         <v>46301.5</v>
       </c>
-      <c r="F7" s="8" t="n">
+      <c r="F7" s="11" t="n">
         <v>46302.54166666666</v>
       </c>
-      <c r="G7" s="9">
+      <c r="G7" s="26">
         <f>(F7-E7)*24</f>
         <v/>
       </c>
-      <c r="H7" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I7" s="7" t="inlineStr"/>
+      <c r="H7" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I7" s="23" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -4373,28 +5238,28 @@
           <t>SAWASDEE DENEB</t>
         </is>
       </c>
-      <c r="C8" s="7" t="n">
+      <c r="C8" s="23" t="n">
         <v>564</v>
       </c>
-      <c r="D8" s="8" t="n">
+      <c r="D8" s="11" t="n">
         <v>46300</v>
       </c>
-      <c r="E8" s="8" t="n">
+      <c r="E8" s="11" t="n">
         <v>46300.5</v>
       </c>
-      <c r="F8" s="8" t="n">
+      <c r="F8" s="11" t="n">
         <v>46302.5</v>
       </c>
-      <c r="G8" s="9">
+      <c r="G8" s="26">
         <f>(F8-E8)*24</f>
         <v/>
       </c>
-      <c r="H8" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I8" s="7" t="inlineStr"/>
+      <c r="H8" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I8" s="23" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -4407,28 +5272,28 @@
           <t>HARI BHUM (Barge)</t>
         </is>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="C9" s="23" t="n">
         <v>259</v>
       </c>
-      <c r="D9" s="8" t="n">
+      <c r="D9" s="11" t="n">
         <v>46298.20833333334</v>
       </c>
-      <c r="E9" s="8" t="n">
+      <c r="E9" s="11" t="n">
         <v>46298.29166666666</v>
       </c>
-      <c r="F9" s="8" t="n">
+      <c r="F9" s="11" t="n">
         <v>46298.66666666666</v>
       </c>
-      <c r="G9" s="9">
+      <c r="G9" s="26">
         <f>(F9-E9)*24</f>
         <v/>
       </c>
-      <c r="H9" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I9" s="7" t="inlineStr"/>
+      <c r="H9" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I9" s="23" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -4441,28 +5306,28 @@
           <t>WAN HAI 278</t>
         </is>
       </c>
-      <c r="C10" s="7" t="n">
+      <c r="C10" s="23" t="n">
         <v>564</v>
       </c>
-      <c r="D10" s="8" t="n">
+      <c r="D10" s="11" t="n">
         <v>46297.91666666666</v>
       </c>
-      <c r="E10" s="8" t="n">
+      <c r="E10" s="11" t="n">
         <v>46298.41666666666</v>
       </c>
-      <c r="F10" s="8" t="n">
+      <c r="F10" s="11" t="n">
         <v>46300.45833333334</v>
       </c>
-      <c r="G10" s="9">
+      <c r="G10" s="26">
         <f>(F10-E10)*24</f>
         <v/>
       </c>
-      <c r="H10" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I10" s="7" t="inlineStr"/>
+      <c r="H10" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I10" s="23" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -4475,28 +5340,28 @@
           <t>KMTC BANGKOK</t>
         </is>
       </c>
-      <c r="C11" s="7" t="n">
+      <c r="C11" s="23" t="n">
         <v>564</v>
       </c>
-      <c r="D11" s="8" t="n">
+      <c r="D11" s="11" t="n">
         <v>46297.29166666666</v>
       </c>
-      <c r="E11" s="8" t="n">
+      <c r="E11" s="11" t="n">
         <v>46297.45833333334</v>
       </c>
-      <c r="F11" s="8" t="n">
+      <c r="F11" s="11" t="n">
         <v>46298.70833333334</v>
       </c>
-      <c r="G11" s="9">
+      <c r="G11" s="26">
         <f>(F11-E11)*24</f>
         <v/>
       </c>
-      <c r="H11" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I11" s="7" t="inlineStr"/>
+      <c r="H11" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I11" s="23" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -4509,28 +5374,28 @@
           <t>XIN MING ZHOU 98</t>
         </is>
       </c>
-      <c r="C12" s="7" t="n">
+      <c r="C12" s="23" t="n">
         <v>564</v>
       </c>
-      <c r="D12" s="8" t="n">
+      <c r="D12" s="11" t="n">
         <v>46299.375</v>
       </c>
-      <c r="E12" s="8" t="n">
+      <c r="E12" s="11" t="n">
         <v>46299.375</v>
       </c>
-      <c r="F12" s="8" t="n">
+      <c r="F12" s="11" t="n">
         <v>46300.375</v>
       </c>
-      <c r="G12" s="9">
+      <c r="G12" s="26">
         <f>(F12-E12)*24</f>
         <v/>
       </c>
-      <c r="H12" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I12" s="7" t="inlineStr"/>
+      <c r="H12" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I12" s="23" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4622,28 +5487,28 @@
           <t>RESURGENCE</t>
         </is>
       </c>
-      <c r="C4" s="7" t="n">
+      <c r="C4" s="23" t="n">
         <v>458</v>
       </c>
-      <c r="D4" s="8" t="n">
+      <c r="D4" s="11" t="n">
         <v>46298.5</v>
       </c>
-      <c r="E4" s="8" t="n">
+      <c r="E4" s="11" t="n">
         <v>46298.5</v>
       </c>
-      <c r="F4" s="8" t="n">
+      <c r="F4" s="11" t="n">
         <v>46299.70833333334</v>
       </c>
-      <c r="G4" s="9">
+      <c r="G4" s="26">
         <f>(F4-E4)*24</f>
         <v/>
       </c>
-      <c r="H4" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I4" s="7" t="inlineStr"/>
+      <c r="H4" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I4" s="23" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -4656,28 +5521,28 @@
           <t>ZHONG GU BEI HAI</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C5" s="23" t="n">
         <v>561</v>
       </c>
-      <c r="D5" s="8" t="n">
+      <c r="D5" s="11" t="n">
         <v>46299.375</v>
       </c>
-      <c r="E5" s="8" t="n">
+      <c r="E5" s="11" t="n">
         <v>46299.625</v>
       </c>
-      <c r="F5" s="8" t="n">
+      <c r="F5" s="11" t="n">
         <v>46301.41666666666</v>
       </c>
-      <c r="G5" s="9">
+      <c r="G5" s="26">
         <f>(F5-E5)*24</f>
         <v/>
       </c>
-      <c r="H5" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I5" s="7" t="inlineStr"/>
+      <c r="H5" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I5" s="23" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -4690,28 +5555,28 @@
           <t>JOSCO LUCKY</t>
         </is>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="23" t="n">
         <v>564</v>
       </c>
-      <c r="D6" s="8" t="n">
+      <c r="D6" s="11" t="n">
         <v>46300.91666666666</v>
       </c>
-      <c r="E6" s="8" t="n">
+      <c r="E6" s="11" t="n">
         <v>46301.5</v>
       </c>
-      <c r="F6" s="8" t="n">
+      <c r="F6" s="11" t="n">
         <v>46302.54166666666</v>
       </c>
-      <c r="G6" s="9">
+      <c r="G6" s="26">
         <f>(F6-E6)*24</f>
         <v/>
       </c>
-      <c r="H6" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I6" s="7" t="inlineStr"/>
+      <c r="H6" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I6" s="23" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -4724,28 +5589,28 @@
           <t>YM IMPROVEMENT</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C7" s="23" t="n">
         <v>564</v>
       </c>
-      <c r="D7" s="8" t="n">
+      <c r="D7" s="11" t="n">
         <v>46298.95833333334</v>
       </c>
-      <c r="E7" s="8" t="n">
+      <c r="E7" s="11" t="n">
         <v>46299.41666666666</v>
       </c>
-      <c r="F7" s="8" t="n">
+      <c r="F7" s="11" t="n">
         <v>46300.5</v>
       </c>
-      <c r="G7" s="9">
+      <c r="G7" s="26">
         <f>(F7-E7)*24</f>
         <v/>
       </c>
-      <c r="H7" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I7" s="7" t="inlineStr"/>
+      <c r="H7" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I7" s="23" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -4758,28 +5623,28 @@
           <t>SAWASDEE SPICA</t>
         </is>
       </c>
-      <c r="C8" s="7" t="n">
+      <c r="C8" s="23" t="n">
         <v>564</v>
       </c>
-      <c r="D8" s="8" t="n">
+      <c r="D8" s="11" t="n">
         <v>46300.875</v>
       </c>
-      <c r="E8" s="8" t="n">
+      <c r="E8" s="11" t="n">
         <v>46301.54166666666</v>
       </c>
-      <c r="F8" s="8" t="n">
+      <c r="F8" s="11" t="n">
         <v>46303.54166666666</v>
       </c>
-      <c r="G8" s="9">
+      <c r="G8" s="26">
         <f>(F8-E8)*24</f>
         <v/>
       </c>
-      <c r="H8" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I8" s="7" t="inlineStr"/>
+      <c r="H8" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I8" s="23" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -4792,28 +5657,28 @@
           <t>SAWASDEE DENEB</t>
         </is>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="C9" s="23" t="n">
         <v>564</v>
       </c>
-      <c r="D9" s="8" t="n">
+      <c r="D9" s="11" t="n">
         <v>46300</v>
       </c>
-      <c r="E9" s="8" t="n">
+      <c r="E9" s="11" t="n">
         <v>46300.5</v>
       </c>
-      <c r="F9" s="8" t="n">
+      <c r="F9" s="11" t="n">
         <v>46302.5</v>
       </c>
-      <c r="G9" s="9">
+      <c r="G9" s="26">
         <f>(F9-E9)*24</f>
         <v/>
       </c>
-      <c r="H9" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I9" s="7" t="inlineStr"/>
+      <c r="H9" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I9" s="23" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -4826,28 +5691,28 @@
           <t>WAN HAI 278</t>
         </is>
       </c>
-      <c r="C10" s="7" t="n">
+      <c r="C10" s="23" t="n">
         <v>564</v>
       </c>
-      <c r="D10" s="8" t="n">
+      <c r="D10" s="11" t="n">
         <v>46297.75</v>
       </c>
-      <c r="E10" s="8" t="n">
+      <c r="E10" s="11" t="n">
         <v>46298.41666666666</v>
       </c>
-      <c r="F10" s="8" t="n">
+      <c r="F10" s="11" t="n">
         <v>46300.45833333334</v>
       </c>
-      <c r="G10" s="9">
+      <c r="G10" s="26">
         <f>(F10-E10)*24</f>
         <v/>
       </c>
-      <c r="H10" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I10" s="7" t="inlineStr"/>
+      <c r="H10" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I10" s="23" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -4860,28 +5725,28 @@
           <t>XIN MING ZHOU 98</t>
         </is>
       </c>
-      <c r="C11" s="7" t="n">
+      <c r="C11" s="23" t="n">
         <v>564</v>
       </c>
-      <c r="D11" s="8" t="n">
+      <c r="D11" s="11" t="n">
         <v>46299.375</v>
       </c>
-      <c r="E11" s="8" t="n">
+      <c r="E11" s="11" t="n">
         <v>46299.375</v>
       </c>
-      <c r="F11" s="8" t="n">
+      <c r="F11" s="11" t="n">
         <v>46300.375</v>
       </c>
-      <c r="G11" s="9">
+      <c r="G11" s="26">
         <f>(F11-E11)*24</f>
         <v/>
       </c>
-      <c r="H11" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I11" s="7" t="inlineStr"/>
+      <c r="H11" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I11" s="23" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -4894,28 +5759,28 @@
           <t>KMTC TOKYO</t>
         </is>
       </c>
-      <c r="C12" s="7" t="n">
+      <c r="C12" s="23" t="n">
         <v>565</v>
       </c>
-      <c r="D12" s="8" t="n">
+      <c r="D12" s="11" t="n">
         <v>46301.58333333334</v>
       </c>
-      <c r="E12" s="8" t="n">
+      <c r="E12" s="11" t="n">
         <v>46301.58333333334</v>
       </c>
-      <c r="F12" s="8" t="n">
+      <c r="F12" s="11" t="n">
         <v>46303.5</v>
       </c>
-      <c r="G12" s="9">
+      <c r="G12" s="26">
         <f>(F12-E12)*24</f>
         <v/>
       </c>
-      <c r="H12" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I12" s="7" t="inlineStr"/>
+      <c r="H12" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I12" s="23" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Excel: add per-day notices block to each day sheet alongside the all-days Berth Notices log
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01-10-2026/PAT_Berth_Window.xlsx
+++ b/01-10-2026/PAT_Berth_Window.xlsx
@@ -33,7 +33,7 @@
     <numFmt numFmtId="166" formatCode="dd-mmm hh:mm"/>
     <numFmt numFmtId="167" formatCode="0.0"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -68,6 +68,12 @@
       <name val="Arial"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="0016324F"/>
+      <sz val="12"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -87,7 +93,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -123,11 +129,55 @@
         <color rgb="00D9D9D9"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -206,6 +256,11 @@
     <xf numFmtId="167" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1465,7 +1520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1919,7 +1974,136 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="28" t="inlineStr">
+        <is>
+          <t>Berth &amp; gate notices on this sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Berth / Gate</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="n"/>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>From</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>To</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Notice / change vs previous sheet</t>
+        </is>
+      </c>
+      <c r="G18" s="29" t="n"/>
+      <c r="H18" s="29" t="n"/>
+      <c r="I18" s="30" t="n"/>
+    </row>
+    <row r="19" ht="42" customHeight="1">
+      <c r="A19" s="16" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="C19" s="32" t="n"/>
+      <c r="D19" s="17" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E19" s="17" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>(no notice – wharf open)  —  Notice removed: 20C reopened on 5 Oct</t>
+        </is>
+      </c>
+      <c r="G19" s="32" t="n"/>
+      <c r="H19" s="32" t="n"/>
+      <c r="I19" s="32" t="n"/>
+    </row>
+    <row r="20" ht="42" customHeight="1">
+      <c r="A20" s="16" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B20" s="16" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="C20" s="32" t="n"/>
+      <c r="D20" s="18" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E20" s="18" t="n">
+        <v>46319</v>
+      </c>
+      <c r="F20" s="16" t="inlineStr">
+        <is>
+          <t>Close on 4–24 Oct 2026 to renovate electric channel (but JOSCO LUCKY and MTT BANGKOK are booked at 20D from 06/18)  —  Unchanged – conflicts with vessel bookings, please confirm</t>
+        </is>
+      </c>
+      <c r="G20" s="32" t="n"/>
+      <c r="H20" s="32" t="n"/>
+      <c r="I20" s="32" t="n"/>
+    </row>
+    <row r="21" ht="42" customHeight="1">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>20E / G.25</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>Gate stopped</t>
+        </is>
+      </c>
+      <c r="C21" s="31" t="n"/>
+      <c r="D21" s="10" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E21" s="10" t="n">
+        <v>46313</v>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>G.25 stops working 5–18 Oct 2026 to change trolley rail  —  Unchanged</t>
+        </is>
+      </c>
+      <c r="G21" s="31" t="n"/>
+      <c r="H21" s="31" t="n"/>
+      <c r="I21" s="31" t="n"/>
+    </row>
   </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="F19:I19"/>
+    <mergeCell ref="F18:I18"/>
+    <mergeCell ref="F21:I21"/>
+    <mergeCell ref="F20:I20"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2896,7 +3080,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3342,7 +3526,104 @@
       </c>
       <c r="I14" s="23" t="inlineStr"/>
     </row>
+    <row r="17">
+      <c r="A17" s="28" t="inlineStr">
+        <is>
+          <t>Berth &amp; gate notices on this sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Berth / Gate</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="n"/>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>From</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>To</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Notice / change vs previous sheet</t>
+        </is>
+      </c>
+      <c r="G18" s="29" t="n"/>
+      <c r="H18" s="29" t="n"/>
+      <c r="I18" s="30" t="n"/>
+    </row>
+    <row r="19" ht="42" customHeight="1">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="C19" s="31" t="n"/>
+      <c r="D19" s="10" t="n">
+        <v>46212</v>
+      </c>
+      <c r="E19" s="10" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F19" s="9" t="inlineStr">
+        <is>
+          <t>20C closed 9 Jul – 30 Sep 2026 (cable track repair)  —  First sheet in the log</t>
+        </is>
+      </c>
+      <c r="G19" s="31" t="n"/>
+      <c r="H19" s="31" t="n"/>
+      <c r="I19" s="31" t="n"/>
+    </row>
+    <row r="20" ht="42" customHeight="1">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>Cable splicing</t>
+        </is>
+      </c>
+      <c r="C20" s="31" t="n"/>
+      <c r="D20" s="11" t="n">
+        <v>46295.35416666666</v>
+      </c>
+      <c r="E20" s="11" t="n">
+        <v>46295.6875</v>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t>20D 30 Sep 08:30–16:30 (cable splicing)  —  First sheet in the log</t>
+        </is>
+      </c>
+      <c r="G20" s="31" t="n"/>
+      <c r="H20" s="31" t="n"/>
+      <c r="I20" s="31" t="n"/>
+    </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="F19:I19"/>
+    <mergeCell ref="F18:I18"/>
+    <mergeCell ref="F20:I20"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3353,7 +3634,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3761,7 +4042,162 @@
       </c>
       <c r="I13" s="23" t="inlineStr"/>
     </row>
+    <row r="16">
+      <c r="A16" s="28" t="inlineStr">
+        <is>
+          <t>Berth &amp; gate notices on this sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Berth / Gate</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="n"/>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>From</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>To</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Notice / change vs previous sheet</t>
+        </is>
+      </c>
+      <c r="G17" s="29" t="n"/>
+      <c r="H17" s="29" t="n"/>
+      <c r="I17" s="30" t="n"/>
+    </row>
+    <row r="18" ht="42" customHeight="1">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>20AB / G.29</t>
+        </is>
+      </c>
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>Gate stopped</t>
+        </is>
+      </c>
+      <c r="C18" s="32" t="n"/>
+      <c r="D18" s="18" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E18" s="18" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F18" s="16" t="inlineStr">
+        <is>
+          <t>G.29 stops working 29–30 Sep 2026 to repair spreader  —  New</t>
+        </is>
+      </c>
+      <c r="G18" s="32" t="n"/>
+      <c r="H18" s="32" t="n"/>
+      <c r="I18" s="32" t="n"/>
+    </row>
+    <row r="19" ht="42" customHeight="1">
+      <c r="A19" s="16" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="C19" s="32" t="n"/>
+      <c r="D19" s="17" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E19" s="18" t="n">
+        <v>46296</v>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>Wharf will be utilised on 1 Oct 2026  —  Reopening moved 30 Sep → 1 Oct</t>
+        </is>
+      </c>
+      <c r="G19" s="32" t="n"/>
+      <c r="H19" s="32" t="n"/>
+      <c r="I19" s="32" t="n"/>
+    </row>
+    <row r="20" ht="42" customHeight="1">
+      <c r="A20" s="16" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B20" s="16" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="C20" s="32" t="n"/>
+      <c r="D20" s="18" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E20" s="18" t="n">
+        <v>46316</v>
+      </c>
+      <c r="F20" s="16" t="inlineStr">
+        <is>
+          <t>Close on 1–21 Oct 2026 to renovate electric channel  —  New (replaces the 30 Sep splicing notice)</t>
+        </is>
+      </c>
+      <c r="G20" s="32" t="n"/>
+      <c r="H20" s="32" t="n"/>
+      <c r="I20" s="32" t="n"/>
+    </row>
+    <row r="21" ht="42" customHeight="1">
+      <c r="A21" s="16" t="inlineStr">
+        <is>
+          <t>20E / G.25</t>
+        </is>
+      </c>
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>Gate stopped</t>
+        </is>
+      </c>
+      <c r="C21" s="32" t="n"/>
+      <c r="D21" s="18" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E21" s="18" t="n">
+        <v>46310</v>
+      </c>
+      <c r="F21" s="16" t="inlineStr">
+        <is>
+          <t>G.25 stops working 1–15 Oct 2026 to change trolley rail  —  New</t>
+        </is>
+      </c>
+      <c r="G21" s="32" t="n"/>
+      <c r="H21" s="32" t="n"/>
+      <c r="I21" s="32" t="n"/>
+    </row>
   </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="F18:I18"/>
+    <mergeCell ref="F17:I17"/>
+    <mergeCell ref="F21:I21"/>
+    <mergeCell ref="F19:I19"/>
+    <mergeCell ref="F20:I20"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3772,7 +4208,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4154,7 +4590,162 @@
       </c>
       <c r="I12" s="23" t="inlineStr"/>
     </row>
+    <row r="15">
+      <c r="A15" s="28" t="inlineStr">
+        <is>
+          <t>Berth &amp; gate notices on this sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Berth / Gate</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="n"/>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>From</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>To</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Notice / change vs previous sheet</t>
+        </is>
+      </c>
+      <c r="G16" s="29" t="n"/>
+      <c r="H16" s="29" t="n"/>
+      <c r="I16" s="30" t="n"/>
+    </row>
+    <row r="17" ht="42" customHeight="1">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>20AB / G.29</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Gate stopped</t>
+        </is>
+      </c>
+      <c r="C17" s="31" t="n"/>
+      <c r="D17" s="10" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E17" s="10" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>G.29 stops working 29–30 Sep 2026 to repair spreader  —  Unchanged</t>
+        </is>
+      </c>
+      <c r="G17" s="31" t="n"/>
+      <c r="H17" s="31" t="n"/>
+      <c r="I17" s="31" t="n"/>
+    </row>
+    <row r="18" ht="42" customHeight="1">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="C18" s="32" t="n"/>
+      <c r="D18" s="17" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E18" s="18" t="n">
+        <v>46298</v>
+      </c>
+      <c r="F18" s="16" t="inlineStr">
+        <is>
+          <t>Wharf will be utilised on 3 Oct 2026  —  Slipped: reopening 1 Oct → 3 Oct</t>
+        </is>
+      </c>
+      <c r="G18" s="32" t="n"/>
+      <c r="H18" s="32" t="n"/>
+      <c r="I18" s="32" t="n"/>
+    </row>
+    <row r="19" ht="42" customHeight="1">
+      <c r="A19" s="16" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="C19" s="32" t="n"/>
+      <c r="D19" s="18" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E19" s="18" t="n">
+        <v>46319</v>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>Close on 3–24 Oct 2026 to renovate electric channel  —  Slipped: 1–21 Oct → 3–24 Oct</t>
+        </is>
+      </c>
+      <c r="G19" s="32" t="n"/>
+      <c r="H19" s="32" t="n"/>
+      <c r="I19" s="32" t="n"/>
+    </row>
+    <row r="20" ht="42" customHeight="1">
+      <c r="A20" s="16" t="inlineStr">
+        <is>
+          <t>20E / G.25</t>
+        </is>
+      </c>
+      <c r="B20" s="16" t="inlineStr">
+        <is>
+          <t>Gate stopped</t>
+        </is>
+      </c>
+      <c r="C20" s="32" t="n"/>
+      <c r="D20" s="18" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E20" s="18" t="n">
+        <v>46313</v>
+      </c>
+      <c r="F20" s="16" t="inlineStr">
+        <is>
+          <t>G.25 stops working 3–18 Oct 2026 to change trolley rail  —  Slipped: 1–15 Oct → 3–18 Oct</t>
+        </is>
+      </c>
+      <c r="G20" s="32" t="n"/>
+      <c r="H20" s="32" t="n"/>
+      <c r="I20" s="32" t="n"/>
+    </row>
   </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="F18:I18"/>
+    <mergeCell ref="F17:I17"/>
+    <mergeCell ref="F16:I16"/>
+    <mergeCell ref="F19:I19"/>
+    <mergeCell ref="F20:I20"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4165,7 +4756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4513,7 +5104,166 @@
       </c>
       <c r="I11" s="23" t="inlineStr"/>
     </row>
+    <row r="14">
+      <c r="A14" s="28" t="inlineStr">
+        <is>
+          <t>Berth &amp; gate notices on this sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Berth / Gate</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="n"/>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>From</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>To</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Notice / change vs previous sheet</t>
+        </is>
+      </c>
+      <c r="G15" s="29" t="n"/>
+      <c r="H15" s="29" t="n"/>
+      <c r="I15" s="30" t="n"/>
+    </row>
+    <row r="16" ht="42" customHeight="1">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>20AB / G.29</t>
+        </is>
+      </c>
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>Gate stopped</t>
+        </is>
+      </c>
+      <c r="C16" s="32" t="n"/>
+      <c r="D16" s="17" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F16" s="16" t="inlineStr">
+        <is>
+          <t>(no longer listed – 29–30 Sep period has ended)  —  Dropped from sheet</t>
+        </is>
+      </c>
+      <c r="G16" s="32" t="n"/>
+      <c r="H16" s="32" t="n"/>
+      <c r="I16" s="32" t="n"/>
+    </row>
+    <row r="17" ht="42" customHeight="1">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="C17" s="31" t="n"/>
+      <c r="D17" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E17" s="10" t="n">
+        <v>46298</v>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>Wharf will be utilised on 3 Oct (sheet prints 2027, treated as a typo)  —  Unchanged</t>
+        </is>
+      </c>
+      <c r="G17" s="31" t="n"/>
+      <c r="H17" s="31" t="n"/>
+      <c r="I17" s="31" t="n"/>
+    </row>
+    <row r="18" ht="42" customHeight="1">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="C18" s="31" t="n"/>
+      <c r="D18" s="10" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E18" s="10" t="n">
+        <v>46319</v>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>Close on 3–24 Oct 2026 to renovate electric channel  —  Unchanged</t>
+        </is>
+      </c>
+      <c r="G18" s="31" t="n"/>
+      <c r="H18" s="31" t="n"/>
+      <c r="I18" s="31" t="n"/>
+    </row>
+    <row r="19" ht="42" customHeight="1">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>20E / G.25</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>Gate stopped</t>
+        </is>
+      </c>
+      <c r="C19" s="31" t="n"/>
+      <c r="D19" s="10" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E19" s="10" t="n">
+        <v>46313</v>
+      </c>
+      <c r="F19" s="9" t="inlineStr">
+        <is>
+          <t>G.25 stops working 3–18 Oct 2026 to change trolley rail  —  Unchanged</t>
+        </is>
+      </c>
+      <c r="G19" s="31" t="n"/>
+      <c r="H19" s="31" t="n"/>
+      <c r="I19" s="31" t="n"/>
+    </row>
   </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="F18:I18"/>
+    <mergeCell ref="F17:I17"/>
+    <mergeCell ref="F15:I15"/>
+    <mergeCell ref="F16:I16"/>
+    <mergeCell ref="F19:I19"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4524,7 +5274,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5008,7 +5758,134 @@
       </c>
       <c r="I15" s="23" t="inlineStr"/>
     </row>
+    <row r="18">
+      <c r="A18" s="28" t="inlineStr">
+        <is>
+          <t>Berth &amp; gate notices on this sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Berth / Gate</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="n"/>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>From</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>To</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Notice / change vs previous sheet</t>
+        </is>
+      </c>
+      <c r="G19" s="29" t="n"/>
+      <c r="H19" s="29" t="n"/>
+      <c r="I19" s="30" t="n"/>
+    </row>
+    <row r="20" ht="42" customHeight="1">
+      <c r="A20" s="16" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B20" s="16" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="C20" s="32" t="n"/>
+      <c r="D20" s="17" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E20" s="18" t="n">
+        <v>46300</v>
+      </c>
+      <c r="F20" s="16" t="inlineStr">
+        <is>
+          <t>Wharf will be utilised on 5 Oct 2026  —  Slipped: reopening 3 Oct → 5 Oct</t>
+        </is>
+      </c>
+      <c r="G20" s="32" t="n"/>
+      <c r="H20" s="32" t="n"/>
+      <c r="I20" s="32" t="n"/>
+    </row>
+    <row r="21" ht="42" customHeight="1">
+      <c r="A21" s="16" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="C21" s="32" t="n"/>
+      <c r="D21" s="18" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E21" s="18" t="n">
+        <v>46319</v>
+      </c>
+      <c r="F21" s="16" t="inlineStr">
+        <is>
+          <t>Close on 4–24 Oct 2026 to renovate electric channel  —  Slipped: start 3 Oct → 4 Oct</t>
+        </is>
+      </c>
+      <c r="G21" s="32" t="n"/>
+      <c r="H21" s="32" t="n"/>
+      <c r="I21" s="32" t="n"/>
+    </row>
+    <row r="22" ht="42" customHeight="1">
+      <c r="A22" s="16" t="inlineStr">
+        <is>
+          <t>20E / G.25</t>
+        </is>
+      </c>
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>Gate stopped</t>
+        </is>
+      </c>
+      <c r="C22" s="32" t="n"/>
+      <c r="D22" s="18" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E22" s="18" t="n">
+        <v>46313</v>
+      </c>
+      <c r="F22" s="16" t="inlineStr">
+        <is>
+          <t>G.25 stops working 5–18 Oct 2026 to change trolley rail  —  Slipped: start 3 Oct → 5 Oct</t>
+        </is>
+      </c>
+      <c r="G22" s="32" t="n"/>
+      <c r="H22" s="32" t="n"/>
+      <c r="I22" s="32" t="n"/>
+    </row>
   </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="F19:I19"/>
+    <mergeCell ref="F20:I20"/>
+    <mergeCell ref="F21:I21"/>
+    <mergeCell ref="F22:I22"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5019,7 +5896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5397,7 +6274,190 @@
       </c>
       <c r="I12" s="23" t="inlineStr"/>
     </row>
+    <row r="15">
+      <c r="A15" s="28" t="inlineStr">
+        <is>
+          <t>Berth &amp; gate notices on this sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Berth / Gate</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="n"/>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>From</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>To</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Notice / change vs previous sheet</t>
+        </is>
+      </c>
+      <c r="G16" s="29" t="n"/>
+      <c r="H16" s="29" t="n"/>
+      <c r="I16" s="30" t="n"/>
+    </row>
+    <row r="17" ht="42" customHeight="1">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="C17" s="31" t="n"/>
+      <c r="D17" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E17" s="10" t="n">
+        <v>46300</v>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>Wharf will be utilised on 5 Oct 2026  —  Unchanged</t>
+        </is>
+      </c>
+      <c r="G17" s="31" t="n"/>
+      <c r="H17" s="31" t="n"/>
+      <c r="I17" s="31" t="n"/>
+    </row>
+    <row r="18" ht="42" customHeight="1">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>Cable splicing</t>
+        </is>
+      </c>
+      <c r="C18" s="32" t="n"/>
+      <c r="D18" s="25" t="n">
+        <v>46299.375</v>
+      </c>
+      <c r="E18" s="25" t="n">
+        <v>46299.5</v>
+      </c>
+      <c r="F18" s="16" t="inlineStr">
+        <is>
+          <t>20C and 20D cable splicing on 4 Oct 2026, 09:00–12:00  —  New (berthing-section sheet)</t>
+        </is>
+      </c>
+      <c r="G18" s="32" t="n"/>
+      <c r="H18" s="32" t="n"/>
+      <c r="I18" s="32" t="n"/>
+    </row>
+    <row r="19" ht="42" customHeight="1">
+      <c r="A19" s="16" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>Cable splicing</t>
+        </is>
+      </c>
+      <c r="C19" s="32" t="n"/>
+      <c r="D19" s="25" t="n">
+        <v>46299.375</v>
+      </c>
+      <c r="E19" s="25" t="n">
+        <v>46299.5</v>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>20C and 20D cable splicing on 4 Oct 2026, 09:00–12:00  —  New (berthing-section sheet)</t>
+        </is>
+      </c>
+      <c r="G19" s="32" t="n"/>
+      <c r="H19" s="32" t="n"/>
+      <c r="I19" s="32" t="n"/>
+    </row>
+    <row r="20" ht="42" customHeight="1">
+      <c r="A20" s="16" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B20" s="16" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="C20" s="32" t="n"/>
+      <c r="D20" s="18" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E20" s="18" t="n">
+        <v>46320</v>
+      </c>
+      <c r="F20" s="16" t="inlineStr">
+        <is>
+          <t>20D closed 4–25 Oct 2026 to renovate electric channel (cable track bays 1700–1800)  —  End moved 24 → 25 Oct (the feeder sheet of the same day still says 24)</t>
+        </is>
+      </c>
+      <c r="G20" s="32" t="n"/>
+      <c r="H20" s="32" t="n"/>
+      <c r="I20" s="32" t="n"/>
+    </row>
+    <row r="21" ht="42" customHeight="1">
+      <c r="A21" s="16" t="inlineStr">
+        <is>
+          <t>20E / G.25</t>
+        </is>
+      </c>
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>Gate stopped</t>
+        </is>
+      </c>
+      <c r="C21" s="32" t="n"/>
+      <c r="D21" s="25" t="n">
+        <v>46300.5</v>
+      </c>
+      <c r="E21" s="18" t="n">
+        <v>46313</v>
+      </c>
+      <c r="F21" s="16" t="inlineStr">
+        <is>
+          <t>G.25 stops working from 5 Oct 12:00 to change trolley rail (bays 700–900); end date is cut off on this sheet, daily sheet says 18 Oct  —  Start time added (12:00); end date unclear</t>
+        </is>
+      </c>
+      <c r="G21" s="32" t="n"/>
+      <c r="H21" s="32" t="n"/>
+      <c r="I21" s="32" t="n"/>
+    </row>
   </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="F18:I18"/>
+    <mergeCell ref="F17:I17"/>
+    <mergeCell ref="F21:I21"/>
+    <mergeCell ref="F16:I16"/>
+    <mergeCell ref="F19:I19"/>
+    <mergeCell ref="F20:I20"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5408,7 +6468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5782,7 +6842,134 @@
       </c>
       <c r="I12" s="23" t="inlineStr"/>
     </row>
+    <row r="15">
+      <c r="A15" s="28" t="inlineStr">
+        <is>
+          <t>Berth &amp; gate notices on this sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Berth / Gate</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="n"/>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>From</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>To</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Notice / change vs previous sheet</t>
+        </is>
+      </c>
+      <c r="G16" s="29" t="n"/>
+      <c r="H16" s="29" t="n"/>
+      <c r="I16" s="30" t="n"/>
+    </row>
+    <row r="17" ht="42" customHeight="1">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="C17" s="31" t="n"/>
+      <c r="D17" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E17" s="10" t="n">
+        <v>46300</v>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>Wharf will be utilised on 5 Oct (sheet prints 2027, treated as a typo)  —  Unchanged</t>
+        </is>
+      </c>
+      <c r="G17" s="31" t="n"/>
+      <c r="H17" s="31" t="n"/>
+      <c r="I17" s="31" t="n"/>
+    </row>
+    <row r="18" ht="42" customHeight="1">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="C18" s="32" t="n"/>
+      <c r="D18" s="18" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E18" s="18" t="n">
+        <v>46319</v>
+      </c>
+      <c r="F18" s="16" t="inlineStr">
+        <is>
+          <t>Close on 4–24 Oct 2026 to renovate electric channel  —  End back to 24 Oct</t>
+        </is>
+      </c>
+      <c r="G18" s="32" t="n"/>
+      <c r="H18" s="32" t="n"/>
+      <c r="I18" s="32" t="n"/>
+    </row>
+    <row r="19" ht="42" customHeight="1">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>20E / G.25</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>Gate stopped</t>
+        </is>
+      </c>
+      <c r="C19" s="31" t="n"/>
+      <c r="D19" s="10" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E19" s="10" t="n">
+        <v>46313</v>
+      </c>
+      <c r="F19" s="9" t="inlineStr">
+        <is>
+          <t>G.25 stops working 5–18 Oct 2026 to change trolley rail  —  End confirmed as 18 Oct</t>
+        </is>
+      </c>
+      <c r="G19" s="31" t="n"/>
+      <c r="H19" s="31" t="n"/>
+      <c r="I19" s="31" t="n"/>
+    </row>
   </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="F19:I19"/>
+    <mergeCell ref="F18:I18"/>
+    <mergeCell ref="F16:I16"/>
+    <mergeCell ref="F17:I17"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Excel: force English month names and Gregorian year in all date cells
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01-10-2026/PAT_Berth_Window.xlsx
+++ b/01-10-2026/PAT_Berth_Window.xlsx
@@ -17,8 +17,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="dd-mmm-yyyy"/>
-    <numFmt numFmtId="165" formatCode="dd-mmm hh:mm"/>
+    <numFmt numFmtId="164" formatCode="[$-409]dd-mmm-yyyy"/>
+    <numFmt numFmtId="165" formatCode="[$-409]dd-mmm hh:mm"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
   <fonts count="7">

</xml_diff>

<commit_message>
Excel: add combined Vessel List by Berth sheet covering all daily sheets
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01-10-2026/PAT_Berth_Window.xlsx
+++ b/01-10-2026/PAT_Berth_Window.xlsx
@@ -16,12 +16,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="[$-409]dd-mmm-yyyy"/>
     <numFmt numFmtId="165" formatCode="[$-409]dd-mmm hh:mm"/>
-    <numFmt numFmtId="166" formatCode="0.0"/>
+    <numFmt numFmtId="166" formatCode="[$-409]dd-mmm-yyyy hh:mm"/>
+    <numFmt numFmtId="167" formatCode="0.0"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -62,6 +63,11 @@
       <color rgb="0016324F"/>
       <sz val="12"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="000000FF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -165,7 +171,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -238,10 +244,41 @@
     <xf numFmtId="165" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -252,13 +289,7 @@
     <xf numFmtId="165" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="165" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -711,16 +742,16 @@
       <c r="C4" s="23" t="n">
         <v>558</v>
       </c>
-      <c r="D4" s="33" t="n">
+      <c r="D4" s="44" t="n">
         <v>46295.875</v>
       </c>
-      <c r="E4" s="33" t="n">
+      <c r="E4" s="44" t="n">
         <v>46296.25</v>
       </c>
-      <c r="F4" s="33" t="n">
+      <c r="F4" s="44" t="n">
         <v>46297.25</v>
       </c>
-      <c r="G4" s="34">
+      <c r="G4" s="28">
         <f>(F4-E4)*24</f>
         <v/>
       </c>
@@ -745,16 +776,16 @@
       <c r="C5" s="23" t="n">
         <v>565</v>
       </c>
-      <c r="D5" s="33" t="n">
+      <c r="D5" s="44" t="n">
         <v>46297.25</v>
       </c>
-      <c r="E5" s="33" t="n">
+      <c r="E5" s="44" t="n">
         <v>46297.33333333334</v>
       </c>
-      <c r="F5" s="33" t="n">
+      <c r="F5" s="44" t="n">
         <v>46298.70833333334</v>
       </c>
-      <c r="G5" s="34">
+      <c r="G5" s="28">
         <f>(F5-E5)*24</f>
         <v/>
       </c>
@@ -779,16 +810,16 @@
       <c r="C6" s="17" t="n">
         <v>482</v>
       </c>
-      <c r="D6" s="35" t="n">
+      <c r="D6" s="45" t="n">
         <v>46296.5</v>
       </c>
-      <c r="E6" s="35" t="n">
+      <c r="E6" s="45" t="n">
         <v>46296.70833333334</v>
       </c>
-      <c r="F6" s="35" t="n">
+      <c r="F6" s="45" t="n">
         <v>46297.70833333334</v>
       </c>
-      <c r="G6" s="36">
+      <c r="G6" s="34">
         <f>(F6-E6)*24</f>
         <v/>
       </c>
@@ -817,16 +848,16 @@
       <c r="C7" s="23" t="n">
         <v>561</v>
       </c>
-      <c r="D7" s="33" t="n">
+      <c r="D7" s="44" t="n">
         <v>46298.91666666666</v>
       </c>
-      <c r="E7" s="33" t="n">
+      <c r="E7" s="44" t="n">
         <v>46299.375</v>
       </c>
-      <c r="F7" s="33" t="n">
+      <c r="F7" s="44" t="n">
         <v>46300.66666666666</v>
       </c>
-      <c r="G7" s="34">
+      <c r="G7" s="28">
         <f>(F7-E7)*24</f>
         <v/>
       </c>
@@ -851,16 +882,16 @@
       <c r="C8" s="23" t="n">
         <v>564</v>
       </c>
-      <c r="D8" s="33" t="n">
+      <c r="D8" s="44" t="n">
         <v>46298.83333333334</v>
       </c>
-      <c r="E8" s="33" t="n">
+      <c r="E8" s="44" t="n">
         <v>46298.83333333334</v>
       </c>
-      <c r="F8" s="33" t="n">
+      <c r="F8" s="44" t="n">
         <v>46300.41666666666</v>
       </c>
-      <c r="G8" s="34">
+      <c r="G8" s="28">
         <f>(F8-E8)*24</f>
         <v/>
       </c>
@@ -885,16 +916,16 @@
       <c r="C9" s="17" t="n">
         <v>537</v>
       </c>
-      <c r="D9" s="35" t="n">
+      <c r="D9" s="45" t="n">
         <v>46296.70833333334</v>
       </c>
-      <c r="E9" s="35" t="n">
+      <c r="E9" s="45" t="n">
         <v>46296.70833333334</v>
       </c>
-      <c r="F9" s="35" t="n">
+      <c r="F9" s="45" t="n">
         <v>46297.70833333334</v>
       </c>
-      <c r="G9" s="36">
+      <c r="G9" s="34">
         <f>(F9-E9)*24</f>
         <v/>
       </c>
@@ -923,16 +954,16 @@
       <c r="C10" s="23" t="n">
         <v>458</v>
       </c>
-      <c r="D10" s="33" t="n">
+      <c r="D10" s="44" t="n">
         <v>46298.75</v>
       </c>
-      <c r="E10" s="33" t="n">
+      <c r="E10" s="44" t="n">
         <v>46298.75</v>
       </c>
-      <c r="F10" s="33" t="n">
+      <c r="F10" s="44" t="n">
         <v>46299.83333333334</v>
       </c>
-      <c r="G10" s="34">
+      <c r="G10" s="28">
         <f>(F10-E10)*24</f>
         <v/>
       </c>
@@ -957,16 +988,16 @@
       <c r="C11" s="23" t="n">
         <v>564</v>
       </c>
-      <c r="D11" s="33" t="n">
+      <c r="D11" s="44" t="n">
         <v>46297.375</v>
       </c>
-      <c r="E11" s="33" t="n">
+      <c r="E11" s="44" t="n">
         <v>46297.375</v>
       </c>
-      <c r="F11" s="33" t="n">
+      <c r="F11" s="44" t="n">
         <v>46299.41666666666</v>
       </c>
-      <c r="G11" s="34">
+      <c r="G11" s="28">
         <f>(F11-E11)*24</f>
         <v/>
       </c>
@@ -978,7 +1009,7 @@
       <c r="I11" s="23" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="28" t="inlineStr">
+      <c r="A14" s="39" t="inlineStr">
         <is>
           <t>Berth &amp; gate notices on this sheet</t>
         </is>
@@ -1011,9 +1042,9 @@
           <t>Notice / change vs previous sheet</t>
         </is>
       </c>
-      <c r="G15" s="29" t="n"/>
-      <c r="H15" s="29" t="n"/>
-      <c r="I15" s="30" t="n"/>
+      <c r="G15" s="40" t="n"/>
+      <c r="H15" s="40" t="n"/>
+      <c r="I15" s="41" t="n"/>
     </row>
     <row r="16" ht="42" customHeight="1">
       <c r="A16" s="16" t="inlineStr">
@@ -1026,7 +1057,7 @@
           <t>Gate stopped</t>
         </is>
       </c>
-      <c r="C16" s="32" t="n"/>
+      <c r="C16" s="43" t="n"/>
       <c r="D16" s="17" t="inlineStr">
         <is>
           <t>–</t>
@@ -1042,9 +1073,9 @@
           <t>(no longer listed – 29–30 Sep period has ended)  —  Dropped from sheet</t>
         </is>
       </c>
-      <c r="G16" s="29" t="n"/>
-      <c r="H16" s="29" t="n"/>
-      <c r="I16" s="30" t="n"/>
+      <c r="G16" s="40" t="n"/>
+      <c r="H16" s="40" t="n"/>
+      <c r="I16" s="41" t="n"/>
     </row>
     <row r="17" ht="42" customHeight="1">
       <c r="A17" s="9" t="inlineStr">
@@ -1057,13 +1088,13 @@
           <t>Berth closed</t>
         </is>
       </c>
-      <c r="C17" s="31" t="n"/>
+      <c r="C17" s="42" t="n"/>
       <c r="D17" s="23" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="E17" s="37" t="n">
+      <c r="E17" s="46" t="n">
         <v>46298</v>
       </c>
       <c r="F17" s="9" t="inlineStr">
@@ -1071,9 +1102,9 @@
           <t>Wharf will be utilised on 3 Oct (sheet prints 2027, treated as a typo)  —  Unchanged</t>
         </is>
       </c>
-      <c r="G17" s="29" t="n"/>
-      <c r="H17" s="29" t="n"/>
-      <c r="I17" s="30" t="n"/>
+      <c r="G17" s="40" t="n"/>
+      <c r="H17" s="40" t="n"/>
+      <c r="I17" s="41" t="n"/>
     </row>
     <row r="18" ht="42" customHeight="1">
       <c r="A18" s="9" t="inlineStr">
@@ -1086,11 +1117,11 @@
           <t>Berth closed</t>
         </is>
       </c>
-      <c r="C18" s="31" t="n"/>
-      <c r="D18" s="37" t="n">
+      <c r="C18" s="42" t="n"/>
+      <c r="D18" s="46" t="n">
         <v>46298</v>
       </c>
-      <c r="E18" s="37" t="n">
+      <c r="E18" s="46" t="n">
         <v>46319</v>
       </c>
       <c r="F18" s="9" t="inlineStr">
@@ -1098,9 +1129,9 @@
           <t>Close on 3–24 Oct 2026 to renovate electric channel  —  Unchanged</t>
         </is>
       </c>
-      <c r="G18" s="29" t="n"/>
-      <c r="H18" s="29" t="n"/>
-      <c r="I18" s="30" t="n"/>
+      <c r="G18" s="40" t="n"/>
+      <c r="H18" s="40" t="n"/>
+      <c r="I18" s="41" t="n"/>
     </row>
     <row r="19" ht="42" customHeight="1">
       <c r="A19" s="9" t="inlineStr">
@@ -1113,11 +1144,11 @@
           <t>Gate stopped</t>
         </is>
       </c>
-      <c r="C19" s="31" t="n"/>
-      <c r="D19" s="37" t="n">
+      <c r="C19" s="42" t="n"/>
+      <c r="D19" s="46" t="n">
         <v>46298</v>
       </c>
-      <c r="E19" s="37" t="n">
+      <c r="E19" s="46" t="n">
         <v>46313</v>
       </c>
       <c r="F19" s="9" t="inlineStr">
@@ -1125,9 +1156,9 @@
           <t>G.25 stops working 3–18 Oct 2026 to change trolley rail  —  Unchanged</t>
         </is>
       </c>
-      <c r="G19" s="29" t="n"/>
-      <c r="H19" s="29" t="n"/>
-      <c r="I19" s="30" t="n"/>
+      <c r="G19" s="40" t="n"/>
+      <c r="H19" s="40" t="n"/>
+      <c r="I19" s="41" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>

<commit_message>
Add 11 Oct 2026 ship movement data, Excel files and history continuity
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01-10-2026/PAT_Berth_Window.xlsx
+++ b/01-10-2026/PAT_Berth_Window.xlsx
@@ -251,6 +251,12 @@
     <xf numFmtId="167" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -261,12 +267,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="167" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -819,7 +819,7 @@
       <c r="F6" s="45" t="n">
         <v>46297.70833333334</v>
       </c>
-      <c r="G6" s="34">
+      <c r="G6" s="30">
         <f>(F6-E6)*24</f>
         <v/>
       </c>
@@ -925,7 +925,7 @@
       <c r="F9" s="45" t="n">
         <v>46297.70833333334</v>
       </c>
-      <c r="G9" s="34">
+      <c r="G9" s="30">
         <f>(F9-E9)*24</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Add 12 Oct 2026 ship movement data, Excel files and history continuity
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01-10-2026/PAT_Berth_Window.xlsx
+++ b/01-10-2026/PAT_Berth_Window.xlsx
@@ -251,22 +251,22 @@
     <xf numFmtId="167" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="167" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -819,7 +819,7 @@
       <c r="F6" s="45" t="n">
         <v>46297.70833333334</v>
       </c>
-      <c r="G6" s="30">
+      <c r="G6" s="34">
         <f>(F6-E6)*24</f>
         <v/>
       </c>
@@ -925,7 +925,7 @@
       <c r="F9" s="45" t="n">
         <v>46297.70833333334</v>
       </c>
-      <c r="G9" s="30">
+      <c r="G9" s="34">
         <f>(F9-E9)*24</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Vessel list: add Waiting for berth (ETA to P.B, hours) before Hours alongside; dashboard and Excel
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01-10-2026/PAT_Berth_Window.xlsx
+++ b/01-10-2026/PAT_Berth_Window.xlsx
@@ -660,7 +660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -669,9 +669,10 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -714,15 +715,20 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
+          <t>Waiting for Berth (h)</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
           <t>Hours Alongside</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Shift</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>Marked</t>
         </is>
@@ -752,15 +758,19 @@
         <v>46297.25</v>
       </c>
       <c r="G4" s="28">
+        <f>(E4-D4)*24</f>
+        <v/>
+      </c>
+      <c r="H4" s="28">
         <f>(F4-E4)*24</f>
         <v/>
       </c>
-      <c r="H4" s="23" t="inlineStr">
+      <c r="I4" s="23" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="I4" s="23" t="inlineStr"/>
+      <c r="J4" s="23" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -786,15 +796,19 @@
         <v>46298.70833333334</v>
       </c>
       <c r="G5" s="28">
+        <f>(E5-D5)*24</f>
+        <v/>
+      </c>
+      <c r="H5" s="28">
         <f>(F5-E5)*24</f>
         <v/>
       </c>
-      <c r="H5" s="23" t="inlineStr">
+      <c r="I5" s="23" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="I5" s="23" t="inlineStr"/>
+      <c r="J5" s="23" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -820,15 +834,19 @@
         <v>46297.70833333334</v>
       </c>
       <c r="G6" s="34">
+        <f>(E6-D6)*24</f>
+        <v/>
+      </c>
+      <c r="H6" s="34">
         <f>(F6-E6)*24</f>
         <v/>
       </c>
-      <c r="H6" s="17" t="inlineStr">
+      <c r="I6" s="17" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="I6" s="17" t="inlineStr">
+      <c r="J6" s="17" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -858,15 +876,19 @@
         <v>46300.66666666666</v>
       </c>
       <c r="G7" s="28">
+        <f>(E7-D7)*24</f>
+        <v/>
+      </c>
+      <c r="H7" s="28">
         <f>(F7-E7)*24</f>
         <v/>
       </c>
-      <c r="H7" s="23" t="inlineStr">
+      <c r="I7" s="23" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="I7" s="23" t="inlineStr"/>
+      <c r="J7" s="23" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -892,15 +914,19 @@
         <v>46300.41666666666</v>
       </c>
       <c r="G8" s="28">
+        <f>(E8-D8)*24</f>
+        <v/>
+      </c>
+      <c r="H8" s="28">
         <f>(F8-E8)*24</f>
         <v/>
       </c>
-      <c r="H8" s="23" t="inlineStr">
+      <c r="I8" s="23" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="I8" s="23" t="inlineStr"/>
+      <c r="J8" s="23" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -926,15 +952,19 @@
         <v>46297.70833333334</v>
       </c>
       <c r="G9" s="34">
+        <f>(E9-D9)*24</f>
+        <v/>
+      </c>
+      <c r="H9" s="34">
         <f>(F9-E9)*24</f>
         <v/>
       </c>
-      <c r="H9" s="17" t="inlineStr">
+      <c r="I9" s="17" t="inlineStr">
         <is>
           <t>1C</t>
         </is>
       </c>
-      <c r="I9" s="17" t="inlineStr">
+      <c r="J9" s="17" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -964,15 +994,19 @@
         <v>46299.83333333334</v>
       </c>
       <c r="G10" s="28">
+        <f>(E10-D10)*24</f>
+        <v/>
+      </c>
+      <c r="H10" s="28">
         <f>(F10-E10)*24</f>
         <v/>
       </c>
-      <c r="H10" s="23" t="inlineStr">
+      <c r="I10" s="23" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="I10" s="23" t="inlineStr"/>
+      <c r="J10" s="23" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -998,15 +1032,19 @@
         <v>46299.41666666666</v>
       </c>
       <c r="G11" s="28">
+        <f>(E11-D11)*24</f>
+        <v/>
+      </c>
+      <c r="H11" s="28">
         <f>(F11-E11)*24</f>
         <v/>
       </c>
-      <c r="H11" s="23" t="inlineStr">
+      <c r="I11" s="23" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="I11" s="23" t="inlineStr"/>
+      <c r="J11" s="23" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="39" t="inlineStr">
@@ -1044,7 +1082,8 @@
       </c>
       <c r="G15" s="40" t="n"/>
       <c r="H15" s="40" t="n"/>
-      <c r="I15" s="41" t="n"/>
+      <c r="I15" s="40" t="n"/>
+      <c r="J15" s="41" t="n"/>
     </row>
     <row r="16" ht="42" customHeight="1">
       <c r="A16" s="16" t="inlineStr">
@@ -1075,7 +1114,8 @@
       </c>
       <c r="G16" s="40" t="n"/>
       <c r="H16" s="40" t="n"/>
-      <c r="I16" s="41" t="n"/>
+      <c r="I16" s="40" t="n"/>
+      <c r="J16" s="41" t="n"/>
     </row>
     <row r="17" ht="42" customHeight="1">
       <c r="A17" s="9" t="inlineStr">
@@ -1104,7 +1144,8 @@
       </c>
       <c r="G17" s="40" t="n"/>
       <c r="H17" s="40" t="n"/>
-      <c r="I17" s="41" t="n"/>
+      <c r="I17" s="40" t="n"/>
+      <c r="J17" s="41" t="n"/>
     </row>
     <row r="18" ht="42" customHeight="1">
       <c r="A18" s="9" t="inlineStr">
@@ -1131,7 +1172,8 @@
       </c>
       <c r="G18" s="40" t="n"/>
       <c r="H18" s="40" t="n"/>
-      <c r="I18" s="41" t="n"/>
+      <c r="I18" s="40" t="n"/>
+      <c r="J18" s="41" t="n"/>
     </row>
     <row r="19" ht="42" customHeight="1">
       <c r="A19" s="9" t="inlineStr">
@@ -1158,15 +1200,16 @@
       </c>
       <c r="G19" s="40" t="n"/>
       <c r="H19" s="40" t="n"/>
-      <c r="I19" s="41" t="n"/>
+      <c r="I19" s="40" t="n"/>
+      <c r="J19" s="41" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="F18:I18"/>
-    <mergeCell ref="F17:I17"/>
-    <mergeCell ref="F15:I15"/>
-    <mergeCell ref="F16:I16"/>
-    <mergeCell ref="F19:I19"/>
+    <mergeCell ref="F17:J17"/>
+    <mergeCell ref="F15:J15"/>
+    <mergeCell ref="F16:J16"/>
+    <mergeCell ref="F19:J19"/>
+    <mergeCell ref="F18:J18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 15 Oct 2026 ship movement data (new sheet layout, berth 20A, 20E closure), Excel and history
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01-10-2026/PAT_Berth_Window.xlsx
+++ b/01-10-2026/PAT_Berth_Window.xlsx
@@ -171,7 +171,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -223,22 +223,7 @@
     <xf numFmtId="164" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -248,6 +233,9 @@
     <xf numFmtId="166" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="167" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -255,6 +243,12 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -269,17 +263,8 @@
     <xf numFmtId="167" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -292,7 +277,7 @@
     <xf numFmtId="165" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -748,20 +733,20 @@
       <c r="C4" s="23" t="n">
         <v>558</v>
       </c>
-      <c r="D4" s="44" t="n">
+      <c r="D4" s="39" t="n">
         <v>46295.875</v>
       </c>
-      <c r="E4" s="44" t="n">
+      <c r="E4" s="39" t="n">
         <v>46296.25</v>
       </c>
-      <c r="F4" s="44" t="n">
+      <c r="F4" s="39" t="n">
         <v>46297.25</v>
       </c>
-      <c r="G4" s="28">
+      <c r="G4" s="24">
         <f>(E4-D4)*24</f>
         <v/>
       </c>
-      <c r="H4" s="28">
+      <c r="H4" s="24">
         <f>(F4-E4)*24</f>
         <v/>
       </c>
@@ -786,20 +771,20 @@
       <c r="C5" s="23" t="n">
         <v>565</v>
       </c>
-      <c r="D5" s="44" t="n">
+      <c r="D5" s="39" t="n">
         <v>46297.25</v>
       </c>
-      <c r="E5" s="44" t="n">
+      <c r="E5" s="39" t="n">
         <v>46297.33333333334</v>
       </c>
-      <c r="F5" s="44" t="n">
+      <c r="F5" s="39" t="n">
         <v>46298.70833333334</v>
       </c>
-      <c r="G5" s="28">
+      <c r="G5" s="24">
         <f>(E5-D5)*24</f>
         <v/>
       </c>
-      <c r="H5" s="28">
+      <c r="H5" s="24">
         <f>(F5-E5)*24</f>
         <v/>
       </c>
@@ -824,20 +809,20 @@
       <c r="C6" s="17" t="n">
         <v>482</v>
       </c>
-      <c r="D6" s="45" t="n">
+      <c r="D6" s="40" t="n">
         <v>46296.5</v>
       </c>
-      <c r="E6" s="45" t="n">
+      <c r="E6" s="40" t="n">
         <v>46296.70833333334</v>
       </c>
-      <c r="F6" s="45" t="n">
+      <c r="F6" s="40" t="n">
         <v>46297.70833333334</v>
       </c>
-      <c r="G6" s="34">
+      <c r="G6" s="32">
         <f>(E6-D6)*24</f>
         <v/>
       </c>
-      <c r="H6" s="34">
+      <c r="H6" s="32">
         <f>(F6-E6)*24</f>
         <v/>
       </c>
@@ -866,20 +851,20 @@
       <c r="C7" s="23" t="n">
         <v>561</v>
       </c>
-      <c r="D7" s="44" t="n">
+      <c r="D7" s="39" t="n">
         <v>46298.91666666666</v>
       </c>
-      <c r="E7" s="44" t="n">
+      <c r="E7" s="39" t="n">
         <v>46299.375</v>
       </c>
-      <c r="F7" s="44" t="n">
+      <c r="F7" s="39" t="n">
         <v>46300.66666666666</v>
       </c>
-      <c r="G7" s="28">
+      <c r="G7" s="24">
         <f>(E7-D7)*24</f>
         <v/>
       </c>
-      <c r="H7" s="28">
+      <c r="H7" s="24">
         <f>(F7-E7)*24</f>
         <v/>
       </c>
@@ -904,20 +889,20 @@
       <c r="C8" s="23" t="n">
         <v>564</v>
       </c>
-      <c r="D8" s="44" t="n">
+      <c r="D8" s="39" t="n">
         <v>46298.83333333334</v>
       </c>
-      <c r="E8" s="44" t="n">
+      <c r="E8" s="39" t="n">
         <v>46298.83333333334</v>
       </c>
-      <c r="F8" s="44" t="n">
+      <c r="F8" s="39" t="n">
         <v>46300.41666666666</v>
       </c>
-      <c r="G8" s="28">
+      <c r="G8" s="24">
         <f>(E8-D8)*24</f>
         <v/>
       </c>
-      <c r="H8" s="28">
+      <c r="H8" s="24">
         <f>(F8-E8)*24</f>
         <v/>
       </c>
@@ -942,20 +927,20 @@
       <c r="C9" s="17" t="n">
         <v>537</v>
       </c>
-      <c r="D9" s="45" t="n">
+      <c r="D9" s="40" t="n">
         <v>46296.70833333334</v>
       </c>
-      <c r="E9" s="45" t="n">
+      <c r="E9" s="40" t="n">
         <v>46296.70833333334</v>
       </c>
-      <c r="F9" s="45" t="n">
+      <c r="F9" s="40" t="n">
         <v>46297.70833333334</v>
       </c>
-      <c r="G9" s="34">
+      <c r="G9" s="32">
         <f>(E9-D9)*24</f>
         <v/>
       </c>
-      <c r="H9" s="34">
+      <c r="H9" s="32">
         <f>(F9-E9)*24</f>
         <v/>
       </c>
@@ -984,20 +969,20 @@
       <c r="C10" s="23" t="n">
         <v>458</v>
       </c>
-      <c r="D10" s="44" t="n">
+      <c r="D10" s="39" t="n">
         <v>46298.75</v>
       </c>
-      <c r="E10" s="44" t="n">
+      <c r="E10" s="39" t="n">
         <v>46298.75</v>
       </c>
-      <c r="F10" s="44" t="n">
+      <c r="F10" s="39" t="n">
         <v>46299.83333333334</v>
       </c>
-      <c r="G10" s="28">
+      <c r="G10" s="24">
         <f>(E10-D10)*24</f>
         <v/>
       </c>
-      <c r="H10" s="28">
+      <c r="H10" s="24">
         <f>(F10-E10)*24</f>
         <v/>
       </c>
@@ -1022,20 +1007,20 @@
       <c r="C11" s="23" t="n">
         <v>564</v>
       </c>
-      <c r="D11" s="44" t="n">
+      <c r="D11" s="39" t="n">
         <v>46297.375</v>
       </c>
-      <c r="E11" s="44" t="n">
+      <c r="E11" s="39" t="n">
         <v>46297.375</v>
       </c>
-      <c r="F11" s="44" t="n">
+      <c r="F11" s="39" t="n">
         <v>46299.41666666666</v>
       </c>
-      <c r="G11" s="28">
+      <c r="G11" s="24">
         <f>(E11-D11)*24</f>
         <v/>
       </c>
-      <c r="H11" s="28">
+      <c r="H11" s="24">
         <f>(F11-E11)*24</f>
         <v/>
       </c>
@@ -1047,7 +1032,7 @@
       <c r="J11" s="23" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="39" t="inlineStr">
+      <c r="A14" s="34" t="inlineStr">
         <is>
           <t>Berth &amp; gate notices on this sheet</t>
         </is>
@@ -1080,10 +1065,10 @@
           <t>Notice / change vs previous sheet</t>
         </is>
       </c>
-      <c r="G15" s="40" t="n"/>
-      <c r="H15" s="40" t="n"/>
-      <c r="I15" s="40" t="n"/>
-      <c r="J15" s="41" t="n"/>
+      <c r="G15" s="35" t="n"/>
+      <c r="H15" s="35" t="n"/>
+      <c r="I15" s="35" t="n"/>
+      <c r="J15" s="36" t="n"/>
     </row>
     <row r="16" ht="42" customHeight="1">
       <c r="A16" s="16" t="inlineStr">
@@ -1096,7 +1081,7 @@
           <t>Gate stopped</t>
         </is>
       </c>
-      <c r="C16" s="43" t="n"/>
+      <c r="C16" s="38" t="n"/>
       <c r="D16" s="17" t="inlineStr">
         <is>
           <t>–</t>
@@ -1112,96 +1097,96 @@
           <t>(no longer listed – 29–30 Sep period has ended)  —  Dropped from sheet</t>
         </is>
       </c>
-      <c r="G16" s="40" t="n"/>
-      <c r="H16" s="40" t="n"/>
-      <c r="I16" s="40" t="n"/>
-      <c r="J16" s="41" t="n"/>
+      <c r="G16" s="35" t="n"/>
+      <c r="H16" s="35" t="n"/>
+      <c r="I16" s="35" t="n"/>
+      <c r="J16" s="36" t="n"/>
     </row>
     <row r="17" ht="42" customHeight="1">
-      <c r="A17" s="9" t="inlineStr">
+      <c r="A17" s="16" t="inlineStr">
         <is>
           <t>20C</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
+      <c r="B17" s="16" t="inlineStr">
         <is>
           <t>Berth closed</t>
         </is>
       </c>
-      <c r="C17" s="42" t="n"/>
-      <c r="D17" s="23" t="inlineStr">
+      <c r="C17" s="38" t="n"/>
+      <c r="D17" s="17" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="E17" s="46" t="n">
+      <c r="E17" s="41" t="n">
         <v>46298</v>
       </c>
-      <c r="F17" s="9" t="inlineStr">
+      <c r="F17" s="16" t="inlineStr">
         <is>
           <t>Wharf will be utilised on 3 Oct (sheet prints 2027, treated as a typo)  —  Unchanged</t>
         </is>
       </c>
-      <c r="G17" s="40" t="n"/>
-      <c r="H17" s="40" t="n"/>
-      <c r="I17" s="40" t="n"/>
-      <c r="J17" s="41" t="n"/>
+      <c r="G17" s="35" t="n"/>
+      <c r="H17" s="35" t="n"/>
+      <c r="I17" s="35" t="n"/>
+      <c r="J17" s="36" t="n"/>
     </row>
     <row r="18" ht="42" customHeight="1">
-      <c r="A18" s="9" t="inlineStr">
+      <c r="A18" s="16" t="inlineStr">
         <is>
           <t>20D</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B18" s="16" t="inlineStr">
         <is>
           <t>Berth closed</t>
         </is>
       </c>
-      <c r="C18" s="42" t="n"/>
-      <c r="D18" s="46" t="n">
+      <c r="C18" s="38" t="n"/>
+      <c r="D18" s="41" t="n">
         <v>46298</v>
       </c>
-      <c r="E18" s="46" t="n">
+      <c r="E18" s="41" t="n">
         <v>46319</v>
       </c>
-      <c r="F18" s="9" t="inlineStr">
+      <c r="F18" s="16" t="inlineStr">
         <is>
           <t>Close on 3–24 Oct 2026 to renovate electric channel  —  Unchanged</t>
         </is>
       </c>
-      <c r="G18" s="40" t="n"/>
-      <c r="H18" s="40" t="n"/>
-      <c r="I18" s="40" t="n"/>
-      <c r="J18" s="41" t="n"/>
+      <c r="G18" s="35" t="n"/>
+      <c r="H18" s="35" t="n"/>
+      <c r="I18" s="35" t="n"/>
+      <c r="J18" s="36" t="n"/>
     </row>
     <row r="19" ht="42" customHeight="1">
-      <c r="A19" s="9" t="inlineStr">
+      <c r="A19" s="16" t="inlineStr">
         <is>
           <t>20E / G.25</t>
         </is>
       </c>
-      <c r="B19" s="9" t="inlineStr">
+      <c r="B19" s="16" t="inlineStr">
         <is>
           <t>Gate stopped</t>
         </is>
       </c>
-      <c r="C19" s="42" t="n"/>
-      <c r="D19" s="46" t="n">
+      <c r="C19" s="38" t="n"/>
+      <c r="D19" s="41" t="n">
         <v>46298</v>
       </c>
-      <c r="E19" s="46" t="n">
+      <c r="E19" s="41" t="n">
         <v>46313</v>
       </c>
-      <c r="F19" s="9" t="inlineStr">
+      <c r="F19" s="16" t="inlineStr">
         <is>
           <t>G.25 stops working 3–18 Oct 2026 to change trolley rail  —  Unchanged</t>
         </is>
       </c>
-      <c r="G19" s="40" t="n"/>
-      <c r="H19" s="40" t="n"/>
-      <c r="I19" s="40" t="n"/>
-      <c r="J19" s="41" t="n"/>
+      <c r="G19" s="35" t="n"/>
+      <c r="H19" s="35" t="n"/>
+      <c r="I19" s="35" t="n"/>
+      <c r="J19" s="36" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>

<commit_message>
Add 20 Oct 2026 ship movement data, Excel files and history continuity
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01-10-2026/PAT_Berth_Window.xlsx
+++ b/01-10-2026/PAT_Berth_Window.xlsx
@@ -22,7 +22,7 @@
     <numFmt numFmtId="166" formatCode="[$-409]dd-mmm-yyyy hh:mm"/>
     <numFmt numFmtId="167" formatCode="0.0"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -65,6 +65,11 @@
     </font>
     <font>
       <name val="Arial"/>
+      <i val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <color rgb="000000FF"/>
       <sz val="10"/>
     </font>
@@ -171,7 +176,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -230,7 +235,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -248,29 +253,30 @@
     <xf numFmtId="164" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="167" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -733,13 +739,13 @@
       <c r="C4" s="23" t="n">
         <v>558</v>
       </c>
-      <c r="D4" s="39" t="n">
+      <c r="D4" s="40" t="n">
         <v>46295.875</v>
       </c>
-      <c r="E4" s="39" t="n">
+      <c r="E4" s="40" t="n">
         <v>46296.25</v>
       </c>
-      <c r="F4" s="39" t="n">
+      <c r="F4" s="40" t="n">
         <v>46297.25</v>
       </c>
       <c r="G4" s="24">
@@ -771,13 +777,13 @@
       <c r="C5" s="23" t="n">
         <v>565</v>
       </c>
-      <c r="D5" s="39" t="n">
+      <c r="D5" s="40" t="n">
         <v>46297.25</v>
       </c>
-      <c r="E5" s="39" t="n">
+      <c r="E5" s="40" t="n">
         <v>46297.33333333334</v>
       </c>
-      <c r="F5" s="39" t="n">
+      <c r="F5" s="40" t="n">
         <v>46298.70833333334</v>
       </c>
       <c r="G5" s="24">
@@ -809,20 +815,20 @@
       <c r="C6" s="17" t="n">
         <v>482</v>
       </c>
-      <c r="D6" s="40" t="n">
+      <c r="D6" s="41" t="n">
         <v>46296.5</v>
       </c>
-      <c r="E6" s="40" t="n">
+      <c r="E6" s="41" t="n">
         <v>46296.70833333334</v>
       </c>
-      <c r="F6" s="40" t="n">
+      <c r="F6" s="41" t="n">
         <v>46297.70833333334</v>
       </c>
-      <c r="G6" s="32">
+      <c r="G6" s="33">
         <f>(E6-D6)*24</f>
         <v/>
       </c>
-      <c r="H6" s="32">
+      <c r="H6" s="33">
         <f>(F6-E6)*24</f>
         <v/>
       </c>
@@ -851,13 +857,13 @@
       <c r="C7" s="23" t="n">
         <v>561</v>
       </c>
-      <c r="D7" s="39" t="n">
+      <c r="D7" s="40" t="n">
         <v>46298.91666666666</v>
       </c>
-      <c r="E7" s="39" t="n">
+      <c r="E7" s="40" t="n">
         <v>46299.375</v>
       </c>
-      <c r="F7" s="39" t="n">
+      <c r="F7" s="40" t="n">
         <v>46300.66666666666</v>
       </c>
       <c r="G7" s="24">
@@ -889,13 +895,13 @@
       <c r="C8" s="23" t="n">
         <v>564</v>
       </c>
-      <c r="D8" s="39" t="n">
+      <c r="D8" s="40" t="n">
         <v>46298.83333333334</v>
       </c>
-      <c r="E8" s="39" t="n">
+      <c r="E8" s="40" t="n">
         <v>46298.83333333334</v>
       </c>
-      <c r="F8" s="39" t="n">
+      <c r="F8" s="40" t="n">
         <v>46300.41666666666</v>
       </c>
       <c r="G8" s="24">
@@ -927,20 +933,20 @@
       <c r="C9" s="17" t="n">
         <v>537</v>
       </c>
-      <c r="D9" s="40" t="n">
+      <c r="D9" s="41" t="n">
         <v>46296.70833333334</v>
       </c>
-      <c r="E9" s="40" t="n">
+      <c r="E9" s="41" t="n">
         <v>46296.70833333334</v>
       </c>
-      <c r="F9" s="40" t="n">
+      <c r="F9" s="41" t="n">
         <v>46297.70833333334</v>
       </c>
-      <c r="G9" s="32">
+      <c r="G9" s="33">
         <f>(E9-D9)*24</f>
         <v/>
       </c>
-      <c r="H9" s="32">
+      <c r="H9" s="33">
         <f>(F9-E9)*24</f>
         <v/>
       </c>
@@ -969,13 +975,13 @@
       <c r="C10" s="23" t="n">
         <v>458</v>
       </c>
-      <c r="D10" s="39" t="n">
+      <c r="D10" s="40" t="n">
         <v>46298.75</v>
       </c>
-      <c r="E10" s="39" t="n">
+      <c r="E10" s="40" t="n">
         <v>46298.75</v>
       </c>
-      <c r="F10" s="39" t="n">
+      <c r="F10" s="40" t="n">
         <v>46299.83333333334</v>
       </c>
       <c r="G10" s="24">
@@ -1007,13 +1013,13 @@
       <c r="C11" s="23" t="n">
         <v>564</v>
       </c>
-      <c r="D11" s="39" t="n">
+      <c r="D11" s="40" t="n">
         <v>46297.375</v>
       </c>
-      <c r="E11" s="39" t="n">
+      <c r="E11" s="40" t="n">
         <v>46297.375</v>
       </c>
-      <c r="F11" s="39" t="n">
+      <c r="F11" s="40" t="n">
         <v>46299.41666666666</v>
       </c>
       <c r="G11" s="24">
@@ -1119,7 +1125,7 @@
           <t>–</t>
         </is>
       </c>
-      <c r="E17" s="41" t="n">
+      <c r="E17" s="42" t="n">
         <v>46298</v>
       </c>
       <c r="F17" s="16" t="inlineStr">
@@ -1144,10 +1150,10 @@
         </is>
       </c>
       <c r="C18" s="38" t="n"/>
-      <c r="D18" s="41" t="n">
+      <c r="D18" s="42" t="n">
         <v>46298</v>
       </c>
-      <c r="E18" s="41" t="n">
+      <c r="E18" s="42" t="n">
         <v>46319</v>
       </c>
       <c r="F18" s="16" t="inlineStr">
@@ -1172,10 +1178,10 @@
         </is>
       </c>
       <c r="C19" s="38" t="n"/>
-      <c r="D19" s="41" t="n">
+      <c r="D19" s="42" t="n">
         <v>46298</v>
       </c>
-      <c r="E19" s="41" t="n">
+      <c r="E19" s="42" t="n">
         <v>46313</v>
       </c>
       <c r="F19" s="16" t="inlineStr">

</xml_diff>

<commit_message>
Add 21 Oct 2026 ship movement data, Excel files and history continuity
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01-10-2026/PAT_Berth_Window.xlsx
+++ b/01-10-2026/PAT_Berth_Window.xlsx
@@ -244,6 +244,12 @@
     <xf numFmtId="167" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -264,12 +270,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -824,11 +824,11 @@
       <c r="F6" s="41" t="n">
         <v>46297.70833333334</v>
       </c>
-      <c r="G6" s="33">
+      <c r="G6" s="26">
         <f>(E6-D6)*24</f>
         <v/>
       </c>
-      <c r="H6" s="33">
+      <c r="H6" s="26">
         <f>(F6-E6)*24</f>
         <v/>
       </c>
@@ -942,11 +942,11 @@
       <c r="F9" s="41" t="n">
         <v>46297.70833333334</v>
       </c>
-      <c r="G9" s="33">
+      <c r="G9" s="26">
         <f>(E9-D9)*24</f>
         <v/>
       </c>
-      <c r="H9" s="33">
+      <c r="H9" s="26">
         <f>(F9-E9)*24</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Add 26 Oct 2026 ship movement data, Excel files and history continuity
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01-10-2026/PAT_Berth_Window.xlsx
+++ b/01-10-2026/PAT_Berth_Window.xlsx
@@ -176,7 +176,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -270,6 +270,15 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -739,13 +748,13 @@
       <c r="C4" s="23" t="n">
         <v>558</v>
       </c>
-      <c r="D4" s="40" t="n">
+      <c r="D4" s="43" t="n">
         <v>46295.875</v>
       </c>
-      <c r="E4" s="40" t="n">
+      <c r="E4" s="43" t="n">
         <v>46296.25</v>
       </c>
-      <c r="F4" s="40" t="n">
+      <c r="F4" s="43" t="n">
         <v>46297.25</v>
       </c>
       <c r="G4" s="24">
@@ -777,13 +786,13 @@
       <c r="C5" s="23" t="n">
         <v>565</v>
       </c>
-      <c r="D5" s="40" t="n">
+      <c r="D5" s="43" t="n">
         <v>46297.25</v>
       </c>
-      <c r="E5" s="40" t="n">
+      <c r="E5" s="43" t="n">
         <v>46297.33333333334</v>
       </c>
-      <c r="F5" s="40" t="n">
+      <c r="F5" s="43" t="n">
         <v>46298.70833333334</v>
       </c>
       <c r="G5" s="24">
@@ -815,13 +824,13 @@
       <c r="C6" s="17" t="n">
         <v>482</v>
       </c>
-      <c r="D6" s="41" t="n">
+      <c r="D6" s="44" t="n">
         <v>46296.5</v>
       </c>
-      <c r="E6" s="41" t="n">
+      <c r="E6" s="44" t="n">
         <v>46296.70833333334</v>
       </c>
-      <c r="F6" s="41" t="n">
+      <c r="F6" s="44" t="n">
         <v>46297.70833333334</v>
       </c>
       <c r="G6" s="26">
@@ -857,13 +866,13 @@
       <c r="C7" s="23" t="n">
         <v>561</v>
       </c>
-      <c r="D7" s="40" t="n">
+      <c r="D7" s="43" t="n">
         <v>46298.91666666666</v>
       </c>
-      <c r="E7" s="40" t="n">
+      <c r="E7" s="43" t="n">
         <v>46299.375</v>
       </c>
-      <c r="F7" s="40" t="n">
+      <c r="F7" s="43" t="n">
         <v>46300.66666666666</v>
       </c>
       <c r="G7" s="24">
@@ -895,13 +904,13 @@
       <c r="C8" s="23" t="n">
         <v>564</v>
       </c>
-      <c r="D8" s="40" t="n">
+      <c r="D8" s="43" t="n">
         <v>46298.83333333334</v>
       </c>
-      <c r="E8" s="40" t="n">
+      <c r="E8" s="43" t="n">
         <v>46298.83333333334</v>
       </c>
-      <c r="F8" s="40" t="n">
+      <c r="F8" s="43" t="n">
         <v>46300.41666666666</v>
       </c>
       <c r="G8" s="24">
@@ -933,13 +942,13 @@
       <c r="C9" s="17" t="n">
         <v>537</v>
       </c>
-      <c r="D9" s="41" t="n">
+      <c r="D9" s="44" t="n">
         <v>46296.70833333334</v>
       </c>
-      <c r="E9" s="41" t="n">
+      <c r="E9" s="44" t="n">
         <v>46296.70833333334</v>
       </c>
-      <c r="F9" s="41" t="n">
+      <c r="F9" s="44" t="n">
         <v>46297.70833333334</v>
       </c>
       <c r="G9" s="26">
@@ -975,13 +984,13 @@
       <c r="C10" s="23" t="n">
         <v>458</v>
       </c>
-      <c r="D10" s="40" t="n">
+      <c r="D10" s="43" t="n">
         <v>46298.75</v>
       </c>
-      <c r="E10" s="40" t="n">
+      <c r="E10" s="43" t="n">
         <v>46298.75</v>
       </c>
-      <c r="F10" s="40" t="n">
+      <c r="F10" s="43" t="n">
         <v>46299.83333333334</v>
       </c>
       <c r="G10" s="24">
@@ -1013,13 +1022,13 @@
       <c r="C11" s="23" t="n">
         <v>564</v>
       </c>
-      <c r="D11" s="40" t="n">
+      <c r="D11" s="43" t="n">
         <v>46297.375</v>
       </c>
-      <c r="E11" s="40" t="n">
+      <c r="E11" s="43" t="n">
         <v>46297.375</v>
       </c>
-      <c r="F11" s="40" t="n">
+      <c r="F11" s="43" t="n">
         <v>46299.41666666666</v>
       </c>
       <c r="G11" s="24">
@@ -1038,7 +1047,7 @@
       <c r="J11" s="23" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="34" t="inlineStr">
+      <c r="A14" s="37" t="inlineStr">
         <is>
           <t>Berth &amp; gate notices on this sheet</t>
         </is>
@@ -1071,10 +1080,10 @@
           <t>Notice / change vs previous sheet</t>
         </is>
       </c>
-      <c r="G15" s="35" t="n"/>
-      <c r="H15" s="35" t="n"/>
-      <c r="I15" s="35" t="n"/>
-      <c r="J15" s="36" t="n"/>
+      <c r="G15" s="38" t="n"/>
+      <c r="H15" s="38" t="n"/>
+      <c r="I15" s="38" t="n"/>
+      <c r="J15" s="39" t="n"/>
     </row>
     <row r="16" ht="42" customHeight="1">
       <c r="A16" s="16" t="inlineStr">
@@ -1087,7 +1096,7 @@
           <t>Gate stopped</t>
         </is>
       </c>
-      <c r="C16" s="38" t="n"/>
+      <c r="C16" s="41" t="n"/>
       <c r="D16" s="17" t="inlineStr">
         <is>
           <t>–</t>
@@ -1103,10 +1112,10 @@
           <t>(no longer listed – 29–30 Sep period has ended)  —  Dropped from sheet</t>
         </is>
       </c>
-      <c r="G16" s="35" t="n"/>
-      <c r="H16" s="35" t="n"/>
-      <c r="I16" s="35" t="n"/>
-      <c r="J16" s="36" t="n"/>
+      <c r="G16" s="38" t="n"/>
+      <c r="H16" s="38" t="n"/>
+      <c r="I16" s="38" t="n"/>
+      <c r="J16" s="39" t="n"/>
     </row>
     <row r="17" ht="42" customHeight="1">
       <c r="A17" s="16" t="inlineStr">
@@ -1119,13 +1128,13 @@
           <t>Berth closed</t>
         </is>
       </c>
-      <c r="C17" s="38" t="n"/>
+      <c r="C17" s="41" t="n"/>
       <c r="D17" s="17" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="E17" s="42" t="n">
+      <c r="E17" s="45" t="n">
         <v>46298</v>
       </c>
       <c r="F17" s="16" t="inlineStr">
@@ -1133,10 +1142,10 @@
           <t>Wharf will be utilised on 3 Oct (sheet prints 2027, treated as a typo)  —  Unchanged</t>
         </is>
       </c>
-      <c r="G17" s="35" t="n"/>
-      <c r="H17" s="35" t="n"/>
-      <c r="I17" s="35" t="n"/>
-      <c r="J17" s="36" t="n"/>
+      <c r="G17" s="38" t="n"/>
+      <c r="H17" s="38" t="n"/>
+      <c r="I17" s="38" t="n"/>
+      <c r="J17" s="39" t="n"/>
     </row>
     <row r="18" ht="42" customHeight="1">
       <c r="A18" s="16" t="inlineStr">
@@ -1149,11 +1158,11 @@
           <t>Berth closed</t>
         </is>
       </c>
-      <c r="C18" s="38" t="n"/>
-      <c r="D18" s="42" t="n">
+      <c r="C18" s="41" t="n"/>
+      <c r="D18" s="45" t="n">
         <v>46298</v>
       </c>
-      <c r="E18" s="42" t="n">
+      <c r="E18" s="45" t="n">
         <v>46319</v>
       </c>
       <c r="F18" s="16" t="inlineStr">
@@ -1161,10 +1170,10 @@
           <t>Close on 3–24 Oct 2026 to renovate electric channel  —  Unchanged</t>
         </is>
       </c>
-      <c r="G18" s="35" t="n"/>
-      <c r="H18" s="35" t="n"/>
-      <c r="I18" s="35" t="n"/>
-      <c r="J18" s="36" t="n"/>
+      <c r="G18" s="38" t="n"/>
+      <c r="H18" s="38" t="n"/>
+      <c r="I18" s="38" t="n"/>
+      <c r="J18" s="39" t="n"/>
     </row>
     <row r="19" ht="42" customHeight="1">
       <c r="A19" s="16" t="inlineStr">
@@ -1177,11 +1186,11 @@
           <t>Gate stopped</t>
         </is>
       </c>
-      <c r="C19" s="38" t="n"/>
-      <c r="D19" s="42" t="n">
+      <c r="C19" s="41" t="n"/>
+      <c r="D19" s="45" t="n">
         <v>46298</v>
       </c>
-      <c r="E19" s="42" t="n">
+      <c r="E19" s="45" t="n">
         <v>46313</v>
       </c>
       <c r="F19" s="16" t="inlineStr">
@@ -1189,10 +1198,10 @@
           <t>G.25 stops working 3–18 Oct 2026 to change trolley rail  —  Unchanged</t>
         </is>
       </c>
-      <c r="G19" s="35" t="n"/>
-      <c r="H19" s="35" t="n"/>
-      <c r="I19" s="35" t="n"/>
-      <c r="J19" s="36" t="n"/>
+      <c r="G19" s="38" t="n"/>
+      <c r="H19" s="38" t="n"/>
+      <c r="I19" s="38" t="n"/>
+      <c r="J19" s="39" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>